<commit_message>
fix: separate game situations from locations
</commit_message>
<xml_diff>
--- a/docs/14-operations/templates/Teelle_New_Game_Template_v2.xlsx
+++ b/docs/14-operations/templates/Teelle_New_Game_Template_v2.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="بازی‌ها" sheetId="1" r:id="R15144b67e7ca4982"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="بازی‌ها" sheetId="1" r:id="Re07cee727bac4938"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -659,7 +659,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="42" t="str">
-        <x:v>هر ردیف یک بازی است. گزینه‌ها را از منوی کشویی انتخاب کنید و متن‌ها را مستقیم در همان خانه بنویسید.</x:v>
+        <x:v>هر ردیف یک بازی است. موقعیت را از میان بعد از کار، روز بارانی یا قبل خواب انتخاب کنید؛ رستوران، ماشین و مهمانی فقط در ستون مکان قرار می‌گیرند.</x:v>
       </x:c>
       <x:c r="B2" s="42"/>
       <x:c r="C2" s="42"/>
@@ -11368,7 +11368,7 @@
       <x:c r="AV204" s="24"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="77">
+  <x:dataValidations count="72">
     <x:dataValidation type="list" sqref="H5:H34">
       <x:formula1>"در دسترس مستقیم,در همان اتاق,بررسی دوره‌ای"</x:formula1>
     </x:dataValidation>
@@ -11408,20 +11408,20 @@
     <x:dataValidation type="list" sqref="Z5:Z34">
       <x:formula1>"بدون آماده‌سازی,ساده,متوسط"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="AA5:AA34">
-      <x:formula1>"ارتباط,بی‌حوصلگی,وقت داخل خانه,بی‌قراری,آرام‌شدن"</x:formula1>
+    <x:dataValidation type="list" allowBlank="1" showDropDown="0" sqref="AA5:AA34">
+      <x:formula1>"بعد از کار,روز بارانی,قبل خواب"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="AB5:AB34">
-      <x:formula1>"ارتباط,بی‌حوصلگی,وقت داخل خانه,بی‌قراری,آرام‌شدن"</x:formula1>
+    <x:dataValidation type="list" allowBlank="1" showDropDown="0" sqref="AB5:AB34">
+      <x:formula1>"بعد از کار,روز بارانی,قبل خواب"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="AC5:AC34">
-      <x:formula1>"ارتباط,بی‌حوصلگی,وقت داخل خانه,بی‌قراری,آرام‌شدن"</x:formula1>
+    <x:dataValidation type="list" allowBlank="1" showDropDown="0" sqref="AC5:AC34">
+      <x:formula1>"بعد از کار,روز بارانی,قبل خواب"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="AD5:AD34">
-      <x:formula1>"داخل خانه,حیاط خانه,سفر,پارک"</x:formula1>
+    <x:dataValidation type="list" allowBlank="1" showDropDown="0" sqref="AD5:AD34">
+      <x:formula1>"داخل خانه,بیرون,رستوران,ماشین,مهمانی"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="AE5:AE34">
-      <x:formula1>"داخل خانه,حیاط خانه,سفر,پارک"</x:formula1>
+    <x:dataValidation type="list" allowBlank="1" showDropDown="0" sqref="AE5:AE34">
+      <x:formula1>"داخل خانه,بیرون,رستوران,ماشین,مهمانی"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AF5:AF34">
       <x:formula1>"آرام,بی‌قرار,هیجان‌زده,غمگین"</x:formula1>
@@ -11537,21 +11537,6 @@
     <x:dataValidation type="list" sqref="Z5:Z204">
       <x:formula1>"بدون آماده‌سازی,ساده,متوسط"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="AA5:AA204">
-      <x:formula1>"بعد از کار,روز بارانی,رستوران,ماشین,مهمانی,قبل خواب"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="AB5:AB204">
-      <x:formula1>"بعد از کار,روز بارانی,رستوران,ماشین,مهمانی,قبل خواب"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="AC5:AC204">
-      <x:formula1>"بعد از کار,روز بارانی,رستوران,ماشین,مهمانی,قبل خواب"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="AD5:AD204">
-      <x:formula1>"داخل خانه,بیرون,رستوران,ماشین,مهمانی"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="AE5:AE204">
-      <x:formula1>"داخل خانه,بیرون,رستوران,ماشین,مهمانی"</x:formula1>
-    </x:dataValidation>
     <x:dataValidation type="list" sqref="AF5:AF204">
       <x:formula1>"آرام,بی‌حوصله,پرانرژی,نیاز به توجه"</x:formula1>
     </x:dataValidation>
@@ -11606,7 +11591,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R641e13e001f3493f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8b30dbac36745cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: finalize daily situation taxonomy
</commit_message>
<xml_diff>
--- a/docs/14-operations/templates/Teelle_New_Game_Template_v2.xlsx
+++ b/docs/14-operations/templates/Teelle_New_Game_Template_v2.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="بازی‌ها" sheetId="1" r:id="Re07cee727bac4938"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="بازی‌ها" sheetId="1" r:id="Rfa7412dd620f4ded"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -61,6 +61,11 @@
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF46676C"/>
+      <x:name val="Vazirmatn"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
       <x:name val="Vazirmatn"/>
     </x:font>
   </x:fonts>
@@ -160,7 +165,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="45">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -270,6 +275,12 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -659,7 +670,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="42" t="str">
-        <x:v>هر ردیف یک بازی است. موقعیت را از میان بعد از کار، روز بارانی یا قبل خواب انتخاب کنید؛ رستوران، ماشین و مهمانی فقط در ستون مکان قرار می‌گیرند.</x:v>
+        <x:v>هر ردیف یک بازی است. موقعیت را فقط از میان بین وعده‌های غذایی، بعد از غذا، بین کارهای روزمره یا قبل از خواب انتخاب کنید. متن انتخاب‌شده در همه منوهای کشویی مشکی نمایش داده می‌شود.</x:v>
       </x:c>
       <x:c r="B2" s="42"/>
       <x:c r="C2" s="42"/>
@@ -1067,58 +1078,58 @@
       <x:c r="E5" s="32" t="str"/>
       <x:c r="F5" s="32" t="str"/>
       <x:c r="G5" s="32" t="str"/>
-      <x:c r="H5" s="32" t="str"/>
-      <x:c r="I5" s="32" t="str"/>
-      <x:c r="J5" s="32" t="str"/>
-      <x:c r="K5" s="32" t="str"/>
-      <x:c r="L5" s="32" t="str"/>
-      <x:c r="M5" s="32" t="str"/>
-      <x:c r="N5" s="32" t="str"/>
-      <x:c r="O5" s="32" t="str"/>
-      <x:c r="P5" s="32" t="str"/>
-      <x:c r="Q5" s="32" t="str"/>
-      <x:c r="R5" s="32" t="str"/>
-      <x:c r="S5" s="32" t="str"/>
-      <x:c r="T5" s="32" t="str"/>
-      <x:c r="U5" s="32" t="str"/>
-      <x:c r="V5" s="32" t="str"/>
-      <x:c r="W5" s="32" t="str"/>
-      <x:c r="X5" s="32" t="str"/>
-      <x:c r="Y5" s="32" t="str"/>
-      <x:c r="Z5" s="32" t="str"/>
-      <x:c r="AA5" s="32" t="str"/>
-      <x:c r="AB5" s="32" t="str"/>
-      <x:c r="AC5" s="32" t="str"/>
-      <x:c r="AD5" s="32" t="str"/>
-      <x:c r="AE5" s="32" t="str"/>
-      <x:c r="AF5" s="32" t="str"/>
-      <x:c r="AG5" s="32" t="str"/>
-      <x:c r="AH5" s="32" t="str"/>
-      <x:c r="AI5" s="32" t="str"/>
-      <x:c r="AJ5" s="32" t="str"/>
-      <x:c r="AK5" s="32" t="str"/>
-      <x:c r="AL5" s="32" t="str"/>
-      <x:c r="AM5" s="32" t="str"/>
+      <x:c r="H5" s="43" t="str"/>
+      <x:c r="I5" s="43" t="str"/>
+      <x:c r="J5" s="43" t="str"/>
+      <x:c r="K5" s="43" t="str"/>
+      <x:c r="L5" s="43" t="str"/>
+      <x:c r="M5" s="43" t="str"/>
+      <x:c r="N5" s="43" t="str"/>
+      <x:c r="O5" s="43" t="str"/>
+      <x:c r="P5" s="43" t="str"/>
+      <x:c r="Q5" s="43" t="str"/>
+      <x:c r="R5" s="43" t="str"/>
+      <x:c r="S5" s="43" t="str"/>
+      <x:c r="T5" s="43" t="str"/>
+      <x:c r="U5" s="43" t="str"/>
+      <x:c r="V5" s="43" t="str"/>
+      <x:c r="W5" s="43" t="str"/>
+      <x:c r="X5" s="43" t="str"/>
+      <x:c r="Y5" s="43" t="str"/>
+      <x:c r="Z5" s="43" t="str"/>
+      <x:c r="AA5" s="43" t="str"/>
+      <x:c r="AB5" s="43" t="str"/>
+      <x:c r="AC5" s="43" t="str"/>
+      <x:c r="AD5" s="43" t="str"/>
+      <x:c r="AE5" s="43" t="str"/>
+      <x:c r="AF5" s="43" t="str"/>
+      <x:c r="AG5" s="43" t="str"/>
+      <x:c r="AH5" s="43" t="str"/>
+      <x:c r="AI5" s="43" t="str"/>
+      <x:c r="AJ5" s="43" t="str"/>
+      <x:c r="AK5" s="43" t="str"/>
+      <x:c r="AL5" s="43" t="str"/>
+      <x:c r="AM5" s="43" t="str"/>
       <x:c r="AN5" s="32" t="str"/>
-      <x:c r="AO5" s="32" t="str"/>
-      <x:c r="AP5" s="32" t="str"/>
+      <x:c r="AO5" s="43" t="str"/>
+      <x:c r="AP5" s="43" t="str"/>
       <x:c r="AQ5" s="32" t="str"/>
-      <x:c r="AR5" s="32" t="str"/>
-      <x:c r="AS5" s="32" t="str"/>
+      <x:c r="AR5" s="43" t="str"/>
+      <x:c r="AS5" s="43" t="str"/>
       <x:c r="AT5" s="32" t="str"/>
       <x:c r="AU5" s="32" t="str"/>
       <x:c r="AV5" s="32" t="str"/>
-      <x:c r="AW5" s="33" t="str"/>
+      <x:c r="AW5" s="44" t="str"/>
       <x:c r="AX5" s="33" t="str"/>
       <x:c r="AY5" s="33" t="str"/>
       <x:c r="AZ5" s="33" t="str"/>
-      <x:c r="BA5" s="33" t="str">
+      <x:c r="BA5" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB5" s="33" t="str">
+      <x:c r="BB5" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC5" s="33" t="str">
+      <x:c r="BC5" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD5" s="33" t="str"/>
@@ -1133,58 +1144,58 @@
       <x:c r="E6" s="32" t="str"/>
       <x:c r="F6" s="32" t="str"/>
       <x:c r="G6" s="32" t="str"/>
-      <x:c r="H6" s="32" t="str"/>
-      <x:c r="I6" s="32" t="str"/>
-      <x:c r="J6" s="32" t="str"/>
-      <x:c r="K6" s="32" t="str"/>
-      <x:c r="L6" s="32" t="str"/>
-      <x:c r="M6" s="32" t="str"/>
-      <x:c r="N6" s="32" t="str"/>
-      <x:c r="O6" s="32" t="str"/>
-      <x:c r="P6" s="32" t="str"/>
-      <x:c r="Q6" s="32" t="str"/>
-      <x:c r="R6" s="32" t="str"/>
-      <x:c r="S6" s="32" t="str"/>
-      <x:c r="T6" s="32" t="str"/>
-      <x:c r="U6" s="32" t="str"/>
-      <x:c r="V6" s="32" t="str"/>
-      <x:c r="W6" s="32" t="str"/>
-      <x:c r="X6" s="32" t="str"/>
-      <x:c r="Y6" s="32" t="str"/>
-      <x:c r="Z6" s="32" t="str"/>
-      <x:c r="AA6" s="32" t="str"/>
-      <x:c r="AB6" s="32" t="str"/>
-      <x:c r="AC6" s="32" t="str"/>
-      <x:c r="AD6" s="32" t="str"/>
-      <x:c r="AE6" s="32" t="str"/>
-      <x:c r="AF6" s="32" t="str"/>
-      <x:c r="AG6" s="32" t="str"/>
-      <x:c r="AH6" s="32" t="str"/>
-      <x:c r="AI6" s="32" t="str"/>
-      <x:c r="AJ6" s="32" t="str"/>
-      <x:c r="AK6" s="32" t="str"/>
-      <x:c r="AL6" s="32" t="str"/>
-      <x:c r="AM6" s="32" t="str"/>
+      <x:c r="H6" s="43" t="str"/>
+      <x:c r="I6" s="43" t="str"/>
+      <x:c r="J6" s="43" t="str"/>
+      <x:c r="K6" s="43" t="str"/>
+      <x:c r="L6" s="43" t="str"/>
+      <x:c r="M6" s="43" t="str"/>
+      <x:c r="N6" s="43" t="str"/>
+      <x:c r="O6" s="43" t="str"/>
+      <x:c r="P6" s="43" t="str"/>
+      <x:c r="Q6" s="43" t="str"/>
+      <x:c r="R6" s="43" t="str"/>
+      <x:c r="S6" s="43" t="str"/>
+      <x:c r="T6" s="43" t="str"/>
+      <x:c r="U6" s="43" t="str"/>
+      <x:c r="V6" s="43" t="str"/>
+      <x:c r="W6" s="43" t="str"/>
+      <x:c r="X6" s="43" t="str"/>
+      <x:c r="Y6" s="43" t="str"/>
+      <x:c r="Z6" s="43" t="str"/>
+      <x:c r="AA6" s="43" t="str"/>
+      <x:c r="AB6" s="43" t="str"/>
+      <x:c r="AC6" s="43" t="str"/>
+      <x:c r="AD6" s="43" t="str"/>
+      <x:c r="AE6" s="43" t="str"/>
+      <x:c r="AF6" s="43" t="str"/>
+      <x:c r="AG6" s="43" t="str"/>
+      <x:c r="AH6" s="43" t="str"/>
+      <x:c r="AI6" s="43" t="str"/>
+      <x:c r="AJ6" s="43" t="str"/>
+      <x:c r="AK6" s="43" t="str"/>
+      <x:c r="AL6" s="43" t="str"/>
+      <x:c r="AM6" s="43" t="str"/>
       <x:c r="AN6" s="32" t="str"/>
-      <x:c r="AO6" s="32" t="str"/>
-      <x:c r="AP6" s="32" t="str"/>
+      <x:c r="AO6" s="43" t="str"/>
+      <x:c r="AP6" s="43" t="str"/>
       <x:c r="AQ6" s="32" t="str"/>
-      <x:c r="AR6" s="32" t="str"/>
-      <x:c r="AS6" s="32" t="str"/>
+      <x:c r="AR6" s="43" t="str"/>
+      <x:c r="AS6" s="43" t="str"/>
       <x:c r="AT6" s="32" t="str"/>
       <x:c r="AU6" s="32" t="str"/>
       <x:c r="AV6" s="32" t="str"/>
-      <x:c r="AW6" s="33" t="str"/>
+      <x:c r="AW6" s="44" t="str"/>
       <x:c r="AX6" s="33" t="str"/>
       <x:c r="AY6" s="33" t="str"/>
       <x:c r="AZ6" s="33" t="str"/>
-      <x:c r="BA6" s="33" t="str">
+      <x:c r="BA6" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB6" s="33" t="str">
+      <x:c r="BB6" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC6" s="33" t="str">
+      <x:c r="BC6" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD6" s="33" t="str"/>
@@ -1199,58 +1210,58 @@
       <x:c r="E7" s="32" t="str"/>
       <x:c r="F7" s="32" t="str"/>
       <x:c r="G7" s="32" t="str"/>
-      <x:c r="H7" s="32" t="str"/>
-      <x:c r="I7" s="32" t="str"/>
-      <x:c r="J7" s="32" t="str"/>
-      <x:c r="K7" s="32" t="str"/>
-      <x:c r="L7" s="32" t="str"/>
-      <x:c r="M7" s="32" t="str"/>
-      <x:c r="N7" s="32" t="str"/>
-      <x:c r="O7" s="32" t="str"/>
-      <x:c r="P7" s="32" t="str"/>
-      <x:c r="Q7" s="32" t="str"/>
-      <x:c r="R7" s="32" t="str"/>
-      <x:c r="S7" s="32" t="str"/>
-      <x:c r="T7" s="32" t="str"/>
-      <x:c r="U7" s="32" t="str"/>
-      <x:c r="V7" s="32" t="str"/>
-      <x:c r="W7" s="32" t="str"/>
-      <x:c r="X7" s="32" t="str"/>
-      <x:c r="Y7" s="32" t="str"/>
-      <x:c r="Z7" s="32" t="str"/>
-      <x:c r="AA7" s="32" t="str"/>
-      <x:c r="AB7" s="32" t="str"/>
-      <x:c r="AC7" s="32" t="str"/>
-      <x:c r="AD7" s="32" t="str"/>
-      <x:c r="AE7" s="32" t="str"/>
-      <x:c r="AF7" s="32" t="str"/>
-      <x:c r="AG7" s="32" t="str"/>
-      <x:c r="AH7" s="32" t="str"/>
-      <x:c r="AI7" s="32" t="str"/>
-      <x:c r="AJ7" s="32" t="str"/>
-      <x:c r="AK7" s="32" t="str"/>
-      <x:c r="AL7" s="32" t="str"/>
-      <x:c r="AM7" s="32" t="str"/>
+      <x:c r="H7" s="43" t="str"/>
+      <x:c r="I7" s="43" t="str"/>
+      <x:c r="J7" s="43" t="str"/>
+      <x:c r="K7" s="43" t="str"/>
+      <x:c r="L7" s="43" t="str"/>
+      <x:c r="M7" s="43" t="str"/>
+      <x:c r="N7" s="43" t="str"/>
+      <x:c r="O7" s="43" t="str"/>
+      <x:c r="P7" s="43" t="str"/>
+      <x:c r="Q7" s="43" t="str"/>
+      <x:c r="R7" s="43" t="str"/>
+      <x:c r="S7" s="43" t="str"/>
+      <x:c r="T7" s="43" t="str"/>
+      <x:c r="U7" s="43" t="str"/>
+      <x:c r="V7" s="43" t="str"/>
+      <x:c r="W7" s="43" t="str"/>
+      <x:c r="X7" s="43" t="str"/>
+      <x:c r="Y7" s="43" t="str"/>
+      <x:c r="Z7" s="43" t="str"/>
+      <x:c r="AA7" s="43" t="str"/>
+      <x:c r="AB7" s="43" t="str"/>
+      <x:c r="AC7" s="43" t="str"/>
+      <x:c r="AD7" s="43" t="str"/>
+      <x:c r="AE7" s="43" t="str"/>
+      <x:c r="AF7" s="43" t="str"/>
+      <x:c r="AG7" s="43" t="str"/>
+      <x:c r="AH7" s="43" t="str"/>
+      <x:c r="AI7" s="43" t="str"/>
+      <x:c r="AJ7" s="43" t="str"/>
+      <x:c r="AK7" s="43" t="str"/>
+      <x:c r="AL7" s="43" t="str"/>
+      <x:c r="AM7" s="43" t="str"/>
       <x:c r="AN7" s="32" t="str"/>
-      <x:c r="AO7" s="32" t="str"/>
-      <x:c r="AP7" s="32" t="str"/>
+      <x:c r="AO7" s="43" t="str"/>
+      <x:c r="AP7" s="43" t="str"/>
       <x:c r="AQ7" s="32" t="str"/>
-      <x:c r="AR7" s="32" t="str"/>
-      <x:c r="AS7" s="32" t="str"/>
+      <x:c r="AR7" s="43" t="str"/>
+      <x:c r="AS7" s="43" t="str"/>
       <x:c r="AT7" s="32" t="str"/>
       <x:c r="AU7" s="32" t="str"/>
       <x:c r="AV7" s="32" t="str"/>
-      <x:c r="AW7" s="33" t="str"/>
+      <x:c r="AW7" s="44" t="str"/>
       <x:c r="AX7" s="33" t="str"/>
       <x:c r="AY7" s="33" t="str"/>
       <x:c r="AZ7" s="33" t="str"/>
-      <x:c r="BA7" s="33" t="str">
+      <x:c r="BA7" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB7" s="33" t="str">
+      <x:c r="BB7" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC7" s="33" t="str">
+      <x:c r="BC7" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD7" s="33" t="str"/>
@@ -1265,58 +1276,58 @@
       <x:c r="E8" s="32" t="str"/>
       <x:c r="F8" s="32" t="str"/>
       <x:c r="G8" s="32" t="str"/>
-      <x:c r="H8" s="32" t="str"/>
-      <x:c r="I8" s="32" t="str"/>
-      <x:c r="J8" s="32" t="str"/>
-      <x:c r="K8" s="32" t="str"/>
-      <x:c r="L8" s="32" t="str"/>
-      <x:c r="M8" s="32" t="str"/>
-      <x:c r="N8" s="32" t="str"/>
-      <x:c r="O8" s="32" t="str"/>
-      <x:c r="P8" s="32" t="str"/>
-      <x:c r="Q8" s="32" t="str"/>
-      <x:c r="R8" s="32" t="str"/>
-      <x:c r="S8" s="32" t="str"/>
-      <x:c r="T8" s="32" t="str"/>
-      <x:c r="U8" s="32" t="str"/>
-      <x:c r="V8" s="32" t="str"/>
-      <x:c r="W8" s="32" t="str"/>
-      <x:c r="X8" s="32" t="str"/>
-      <x:c r="Y8" s="32" t="str"/>
-      <x:c r="Z8" s="32" t="str"/>
-      <x:c r="AA8" s="32" t="str"/>
-      <x:c r="AB8" s="32" t="str"/>
-      <x:c r="AC8" s="32" t="str"/>
-      <x:c r="AD8" s="32" t="str"/>
-      <x:c r="AE8" s="32" t="str"/>
-      <x:c r="AF8" s="32" t="str"/>
-      <x:c r="AG8" s="32" t="str"/>
-      <x:c r="AH8" s="32" t="str"/>
-      <x:c r="AI8" s="32" t="str"/>
-      <x:c r="AJ8" s="32" t="str"/>
-      <x:c r="AK8" s="32" t="str"/>
-      <x:c r="AL8" s="32" t="str"/>
-      <x:c r="AM8" s="32" t="str"/>
+      <x:c r="H8" s="43" t="str"/>
+      <x:c r="I8" s="43" t="str"/>
+      <x:c r="J8" s="43" t="str"/>
+      <x:c r="K8" s="43" t="str"/>
+      <x:c r="L8" s="43" t="str"/>
+      <x:c r="M8" s="43" t="str"/>
+      <x:c r="N8" s="43" t="str"/>
+      <x:c r="O8" s="43" t="str"/>
+      <x:c r="P8" s="43" t="str"/>
+      <x:c r="Q8" s="43" t="str"/>
+      <x:c r="R8" s="43" t="str"/>
+      <x:c r="S8" s="43" t="str"/>
+      <x:c r="T8" s="43" t="str"/>
+      <x:c r="U8" s="43" t="str"/>
+      <x:c r="V8" s="43" t="str"/>
+      <x:c r="W8" s="43" t="str"/>
+      <x:c r="X8" s="43" t="str"/>
+      <x:c r="Y8" s="43" t="str"/>
+      <x:c r="Z8" s="43" t="str"/>
+      <x:c r="AA8" s="43" t="str"/>
+      <x:c r="AB8" s="43" t="str"/>
+      <x:c r="AC8" s="43" t="str"/>
+      <x:c r="AD8" s="43" t="str"/>
+      <x:c r="AE8" s="43" t="str"/>
+      <x:c r="AF8" s="43" t="str"/>
+      <x:c r="AG8" s="43" t="str"/>
+      <x:c r="AH8" s="43" t="str"/>
+      <x:c r="AI8" s="43" t="str"/>
+      <x:c r="AJ8" s="43" t="str"/>
+      <x:c r="AK8" s="43" t="str"/>
+      <x:c r="AL8" s="43" t="str"/>
+      <x:c r="AM8" s="43" t="str"/>
       <x:c r="AN8" s="32" t="str"/>
-      <x:c r="AO8" s="32" t="str"/>
-      <x:c r="AP8" s="32" t="str"/>
+      <x:c r="AO8" s="43" t="str"/>
+      <x:c r="AP8" s="43" t="str"/>
       <x:c r="AQ8" s="32" t="str"/>
-      <x:c r="AR8" s="32" t="str"/>
-      <x:c r="AS8" s="32" t="str"/>
+      <x:c r="AR8" s="43" t="str"/>
+      <x:c r="AS8" s="43" t="str"/>
       <x:c r="AT8" s="32" t="str"/>
       <x:c r="AU8" s="32" t="str"/>
       <x:c r="AV8" s="32" t="str"/>
-      <x:c r="AW8" s="33" t="str"/>
+      <x:c r="AW8" s="44" t="str"/>
       <x:c r="AX8" s="33" t="str"/>
       <x:c r="AY8" s="33" t="str"/>
       <x:c r="AZ8" s="33" t="str"/>
-      <x:c r="BA8" s="33" t="str">
+      <x:c r="BA8" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB8" s="33" t="str">
+      <x:c r="BB8" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC8" s="33" t="str">
+      <x:c r="BC8" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD8" s="33" t="str"/>
@@ -1331,58 +1342,58 @@
       <x:c r="E9" s="32" t="str"/>
       <x:c r="F9" s="32" t="str"/>
       <x:c r="G9" s="32" t="str"/>
-      <x:c r="H9" s="32" t="str"/>
-      <x:c r="I9" s="32" t="str"/>
-      <x:c r="J9" s="32" t="str"/>
-      <x:c r="K9" s="32" t="str"/>
-      <x:c r="L9" s="32" t="str"/>
-      <x:c r="M9" s="32" t="str"/>
-      <x:c r="N9" s="32" t="str"/>
-      <x:c r="O9" s="32" t="str"/>
-      <x:c r="P9" s="32" t="str"/>
-      <x:c r="Q9" s="32" t="str"/>
-      <x:c r="R9" s="32" t="str"/>
-      <x:c r="S9" s="32" t="str"/>
-      <x:c r="T9" s="32" t="str"/>
-      <x:c r="U9" s="32" t="str"/>
-      <x:c r="V9" s="32" t="str"/>
-      <x:c r="W9" s="32" t="str"/>
-      <x:c r="X9" s="32" t="str"/>
-      <x:c r="Y9" s="32" t="str"/>
-      <x:c r="Z9" s="32" t="str"/>
-      <x:c r="AA9" s="32" t="str"/>
-      <x:c r="AB9" s="32" t="str"/>
-      <x:c r="AC9" s="32" t="str"/>
-      <x:c r="AD9" s="32" t="str"/>
-      <x:c r="AE9" s="32" t="str"/>
-      <x:c r="AF9" s="32" t="str"/>
-      <x:c r="AG9" s="32" t="str"/>
-      <x:c r="AH9" s="32" t="str"/>
-      <x:c r="AI9" s="32" t="str"/>
-      <x:c r="AJ9" s="32" t="str"/>
-      <x:c r="AK9" s="32" t="str"/>
-      <x:c r="AL9" s="32" t="str"/>
-      <x:c r="AM9" s="32" t="str"/>
+      <x:c r="H9" s="43" t="str"/>
+      <x:c r="I9" s="43" t="str"/>
+      <x:c r="J9" s="43" t="str"/>
+      <x:c r="K9" s="43" t="str"/>
+      <x:c r="L9" s="43" t="str"/>
+      <x:c r="M9" s="43" t="str"/>
+      <x:c r="N9" s="43" t="str"/>
+      <x:c r="O9" s="43" t="str"/>
+      <x:c r="P9" s="43" t="str"/>
+      <x:c r="Q9" s="43" t="str"/>
+      <x:c r="R9" s="43" t="str"/>
+      <x:c r="S9" s="43" t="str"/>
+      <x:c r="T9" s="43" t="str"/>
+      <x:c r="U9" s="43" t="str"/>
+      <x:c r="V9" s="43" t="str"/>
+      <x:c r="W9" s="43" t="str"/>
+      <x:c r="X9" s="43" t="str"/>
+      <x:c r="Y9" s="43" t="str"/>
+      <x:c r="Z9" s="43" t="str"/>
+      <x:c r="AA9" s="43" t="str"/>
+      <x:c r="AB9" s="43" t="str"/>
+      <x:c r="AC9" s="43" t="str"/>
+      <x:c r="AD9" s="43" t="str"/>
+      <x:c r="AE9" s="43" t="str"/>
+      <x:c r="AF9" s="43" t="str"/>
+      <x:c r="AG9" s="43" t="str"/>
+      <x:c r="AH9" s="43" t="str"/>
+      <x:c r="AI9" s="43" t="str"/>
+      <x:c r="AJ9" s="43" t="str"/>
+      <x:c r="AK9" s="43" t="str"/>
+      <x:c r="AL9" s="43" t="str"/>
+      <x:c r="AM9" s="43" t="str"/>
       <x:c r="AN9" s="32" t="str"/>
-      <x:c r="AO9" s="32" t="str"/>
-      <x:c r="AP9" s="32" t="str"/>
+      <x:c r="AO9" s="43" t="str"/>
+      <x:c r="AP9" s="43" t="str"/>
       <x:c r="AQ9" s="32" t="str"/>
-      <x:c r="AR9" s="32" t="str"/>
-      <x:c r="AS9" s="32" t="str"/>
+      <x:c r="AR9" s="43" t="str"/>
+      <x:c r="AS9" s="43" t="str"/>
       <x:c r="AT9" s="32" t="str"/>
       <x:c r="AU9" s="32" t="str"/>
       <x:c r="AV9" s="32" t="str"/>
-      <x:c r="AW9" s="33" t="str"/>
+      <x:c r="AW9" s="44" t="str"/>
       <x:c r="AX9" s="33" t="str"/>
       <x:c r="AY9" s="33" t="str"/>
       <x:c r="AZ9" s="33" t="str"/>
-      <x:c r="BA9" s="33" t="str">
+      <x:c r="BA9" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB9" s="33" t="str">
+      <x:c r="BB9" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC9" s="33" t="str">
+      <x:c r="BC9" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD9" s="33" t="str"/>
@@ -1397,58 +1408,58 @@
       <x:c r="E10" s="32" t="str"/>
       <x:c r="F10" s="32" t="str"/>
       <x:c r="G10" s="32" t="str"/>
-      <x:c r="H10" s="32" t="str"/>
-      <x:c r="I10" s="32" t="str"/>
-      <x:c r="J10" s="32" t="str"/>
-      <x:c r="K10" s="32" t="str"/>
-      <x:c r="L10" s="32" t="str"/>
-      <x:c r="M10" s="32" t="str"/>
-      <x:c r="N10" s="32" t="str"/>
-      <x:c r="O10" s="32" t="str"/>
-      <x:c r="P10" s="32" t="str"/>
-      <x:c r="Q10" s="32" t="str"/>
-      <x:c r="R10" s="32" t="str"/>
-      <x:c r="S10" s="32" t="str"/>
-      <x:c r="T10" s="32" t="str"/>
-      <x:c r="U10" s="32" t="str"/>
-      <x:c r="V10" s="32" t="str"/>
-      <x:c r="W10" s="32" t="str"/>
-      <x:c r="X10" s="32" t="str"/>
-      <x:c r="Y10" s="32" t="str"/>
-      <x:c r="Z10" s="32" t="str"/>
-      <x:c r="AA10" s="32" t="str"/>
-      <x:c r="AB10" s="32" t="str"/>
-      <x:c r="AC10" s="32" t="str"/>
-      <x:c r="AD10" s="32" t="str"/>
-      <x:c r="AE10" s="32" t="str"/>
-      <x:c r="AF10" s="32" t="str"/>
-      <x:c r="AG10" s="32" t="str"/>
-      <x:c r="AH10" s="32" t="str"/>
-      <x:c r="AI10" s="32" t="str"/>
-      <x:c r="AJ10" s="32" t="str"/>
-      <x:c r="AK10" s="32" t="str"/>
-      <x:c r="AL10" s="32" t="str"/>
-      <x:c r="AM10" s="32" t="str"/>
+      <x:c r="H10" s="43" t="str"/>
+      <x:c r="I10" s="43" t="str"/>
+      <x:c r="J10" s="43" t="str"/>
+      <x:c r="K10" s="43" t="str"/>
+      <x:c r="L10" s="43" t="str"/>
+      <x:c r="M10" s="43" t="str"/>
+      <x:c r="N10" s="43" t="str"/>
+      <x:c r="O10" s="43" t="str"/>
+      <x:c r="P10" s="43" t="str"/>
+      <x:c r="Q10" s="43" t="str"/>
+      <x:c r="R10" s="43" t="str"/>
+      <x:c r="S10" s="43" t="str"/>
+      <x:c r="T10" s="43" t="str"/>
+      <x:c r="U10" s="43" t="str"/>
+      <x:c r="V10" s="43" t="str"/>
+      <x:c r="W10" s="43" t="str"/>
+      <x:c r="X10" s="43" t="str"/>
+      <x:c r="Y10" s="43" t="str"/>
+      <x:c r="Z10" s="43" t="str"/>
+      <x:c r="AA10" s="43" t="str"/>
+      <x:c r="AB10" s="43" t="str"/>
+      <x:c r="AC10" s="43" t="str"/>
+      <x:c r="AD10" s="43" t="str"/>
+      <x:c r="AE10" s="43" t="str"/>
+      <x:c r="AF10" s="43" t="str"/>
+      <x:c r="AG10" s="43" t="str"/>
+      <x:c r="AH10" s="43" t="str"/>
+      <x:c r="AI10" s="43" t="str"/>
+      <x:c r="AJ10" s="43" t="str"/>
+      <x:c r="AK10" s="43" t="str"/>
+      <x:c r="AL10" s="43" t="str"/>
+      <x:c r="AM10" s="43" t="str"/>
       <x:c r="AN10" s="32" t="str"/>
-      <x:c r="AO10" s="32" t="str"/>
-      <x:c r="AP10" s="32" t="str"/>
+      <x:c r="AO10" s="43" t="str"/>
+      <x:c r="AP10" s="43" t="str"/>
       <x:c r="AQ10" s="32" t="str"/>
-      <x:c r="AR10" s="32" t="str"/>
-      <x:c r="AS10" s="32" t="str"/>
+      <x:c r="AR10" s="43" t="str"/>
+      <x:c r="AS10" s="43" t="str"/>
       <x:c r="AT10" s="32" t="str"/>
       <x:c r="AU10" s="32" t="str"/>
       <x:c r="AV10" s="32" t="str"/>
-      <x:c r="AW10" s="33" t="str"/>
+      <x:c r="AW10" s="44" t="str"/>
       <x:c r="AX10" s="33" t="str"/>
       <x:c r="AY10" s="33" t="str"/>
       <x:c r="AZ10" s="33" t="str"/>
-      <x:c r="BA10" s="33" t="str">
+      <x:c r="BA10" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB10" s="33" t="str">
+      <x:c r="BB10" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC10" s="33" t="str">
+      <x:c r="BC10" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD10" s="33" t="str"/>
@@ -1463,58 +1474,58 @@
       <x:c r="E11" s="32" t="str"/>
       <x:c r="F11" s="32" t="str"/>
       <x:c r="G11" s="32" t="str"/>
-      <x:c r="H11" s="32" t="str"/>
-      <x:c r="I11" s="32" t="str"/>
-      <x:c r="J11" s="32" t="str"/>
-      <x:c r="K11" s="32" t="str"/>
-      <x:c r="L11" s="32" t="str"/>
-      <x:c r="M11" s="32" t="str"/>
-      <x:c r="N11" s="32" t="str"/>
-      <x:c r="O11" s="32" t="str"/>
-      <x:c r="P11" s="32" t="str"/>
-      <x:c r="Q11" s="32" t="str"/>
-      <x:c r="R11" s="32" t="str"/>
-      <x:c r="S11" s="32" t="str"/>
-      <x:c r="T11" s="32" t="str"/>
-      <x:c r="U11" s="32" t="str"/>
-      <x:c r="V11" s="32" t="str"/>
-      <x:c r="W11" s="32" t="str"/>
-      <x:c r="X11" s="32" t="str"/>
-      <x:c r="Y11" s="32" t="str"/>
-      <x:c r="Z11" s="32" t="str"/>
-      <x:c r="AA11" s="32" t="str"/>
-      <x:c r="AB11" s="32" t="str"/>
-      <x:c r="AC11" s="32" t="str"/>
-      <x:c r="AD11" s="32" t="str"/>
-      <x:c r="AE11" s="32" t="str"/>
-      <x:c r="AF11" s="32" t="str"/>
-      <x:c r="AG11" s="32" t="str"/>
-      <x:c r="AH11" s="32" t="str"/>
-      <x:c r="AI11" s="32" t="str"/>
-      <x:c r="AJ11" s="32" t="str"/>
-      <x:c r="AK11" s="32" t="str"/>
-      <x:c r="AL11" s="32" t="str"/>
-      <x:c r="AM11" s="32" t="str"/>
+      <x:c r="H11" s="43" t="str"/>
+      <x:c r="I11" s="43" t="str"/>
+      <x:c r="J11" s="43" t="str"/>
+      <x:c r="K11" s="43" t="str"/>
+      <x:c r="L11" s="43" t="str"/>
+      <x:c r="M11" s="43" t="str"/>
+      <x:c r="N11" s="43" t="str"/>
+      <x:c r="O11" s="43" t="str"/>
+      <x:c r="P11" s="43" t="str"/>
+      <x:c r="Q11" s="43" t="str"/>
+      <x:c r="R11" s="43" t="str"/>
+      <x:c r="S11" s="43" t="str"/>
+      <x:c r="T11" s="43" t="str"/>
+      <x:c r="U11" s="43" t="str"/>
+      <x:c r="V11" s="43" t="str"/>
+      <x:c r="W11" s="43" t="str"/>
+      <x:c r="X11" s="43" t="str"/>
+      <x:c r="Y11" s="43" t="str"/>
+      <x:c r="Z11" s="43" t="str"/>
+      <x:c r="AA11" s="43" t="str"/>
+      <x:c r="AB11" s="43" t="str"/>
+      <x:c r="AC11" s="43" t="str"/>
+      <x:c r="AD11" s="43" t="str"/>
+      <x:c r="AE11" s="43" t="str"/>
+      <x:c r="AF11" s="43" t="str"/>
+      <x:c r="AG11" s="43" t="str"/>
+      <x:c r="AH11" s="43" t="str"/>
+      <x:c r="AI11" s="43" t="str"/>
+      <x:c r="AJ11" s="43" t="str"/>
+      <x:c r="AK11" s="43" t="str"/>
+      <x:c r="AL11" s="43" t="str"/>
+      <x:c r="AM11" s="43" t="str"/>
       <x:c r="AN11" s="32" t="str"/>
-      <x:c r="AO11" s="32" t="str"/>
-      <x:c r="AP11" s="32" t="str"/>
+      <x:c r="AO11" s="43" t="str"/>
+      <x:c r="AP11" s="43" t="str"/>
       <x:c r="AQ11" s="32" t="str"/>
-      <x:c r="AR11" s="32" t="str"/>
-      <x:c r="AS11" s="32" t="str"/>
+      <x:c r="AR11" s="43" t="str"/>
+      <x:c r="AS11" s="43" t="str"/>
       <x:c r="AT11" s="32" t="str"/>
       <x:c r="AU11" s="32" t="str"/>
       <x:c r="AV11" s="32" t="str"/>
-      <x:c r="AW11" s="33" t="str"/>
+      <x:c r="AW11" s="44" t="str"/>
       <x:c r="AX11" s="33" t="str"/>
       <x:c r="AY11" s="33" t="str"/>
       <x:c r="AZ11" s="33" t="str"/>
-      <x:c r="BA11" s="33" t="str">
+      <x:c r="BA11" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB11" s="33" t="str">
+      <x:c r="BB11" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC11" s="33" t="str">
+      <x:c r="BC11" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD11" s="33" t="str"/>
@@ -1529,58 +1540,58 @@
       <x:c r="E12" s="32" t="str"/>
       <x:c r="F12" s="32" t="str"/>
       <x:c r="G12" s="32" t="str"/>
-      <x:c r="H12" s="32" t="str"/>
-      <x:c r="I12" s="32" t="str"/>
-      <x:c r="J12" s="32" t="str"/>
-      <x:c r="K12" s="32" t="str"/>
-      <x:c r="L12" s="32" t="str"/>
-      <x:c r="M12" s="32" t="str"/>
-      <x:c r="N12" s="32" t="str"/>
-      <x:c r="O12" s="32" t="str"/>
-      <x:c r="P12" s="32" t="str"/>
-      <x:c r="Q12" s="32" t="str"/>
-      <x:c r="R12" s="32" t="str"/>
-      <x:c r="S12" s="32" t="str"/>
-      <x:c r="T12" s="32" t="str"/>
-      <x:c r="U12" s="32" t="str"/>
-      <x:c r="V12" s="32" t="str"/>
-      <x:c r="W12" s="32" t="str"/>
-      <x:c r="X12" s="32" t="str"/>
-      <x:c r="Y12" s="32" t="str"/>
-      <x:c r="Z12" s="32" t="str"/>
-      <x:c r="AA12" s="32" t="str"/>
-      <x:c r="AB12" s="32" t="str"/>
-      <x:c r="AC12" s="32" t="str"/>
-      <x:c r="AD12" s="32" t="str"/>
-      <x:c r="AE12" s="32" t="str"/>
-      <x:c r="AF12" s="32" t="str"/>
-      <x:c r="AG12" s="32" t="str"/>
-      <x:c r="AH12" s="32" t="str"/>
-      <x:c r="AI12" s="32" t="str"/>
-      <x:c r="AJ12" s="32" t="str"/>
-      <x:c r="AK12" s="32" t="str"/>
-      <x:c r="AL12" s="32" t="str"/>
-      <x:c r="AM12" s="32" t="str"/>
+      <x:c r="H12" s="43" t="str"/>
+      <x:c r="I12" s="43" t="str"/>
+      <x:c r="J12" s="43" t="str"/>
+      <x:c r="K12" s="43" t="str"/>
+      <x:c r="L12" s="43" t="str"/>
+      <x:c r="M12" s="43" t="str"/>
+      <x:c r="N12" s="43" t="str"/>
+      <x:c r="O12" s="43" t="str"/>
+      <x:c r="P12" s="43" t="str"/>
+      <x:c r="Q12" s="43" t="str"/>
+      <x:c r="R12" s="43" t="str"/>
+      <x:c r="S12" s="43" t="str"/>
+      <x:c r="T12" s="43" t="str"/>
+      <x:c r="U12" s="43" t="str"/>
+      <x:c r="V12" s="43" t="str"/>
+      <x:c r="W12" s="43" t="str"/>
+      <x:c r="X12" s="43" t="str"/>
+      <x:c r="Y12" s="43" t="str"/>
+      <x:c r="Z12" s="43" t="str"/>
+      <x:c r="AA12" s="43" t="str"/>
+      <x:c r="AB12" s="43" t="str"/>
+      <x:c r="AC12" s="43" t="str"/>
+      <x:c r="AD12" s="43" t="str"/>
+      <x:c r="AE12" s="43" t="str"/>
+      <x:c r="AF12" s="43" t="str"/>
+      <x:c r="AG12" s="43" t="str"/>
+      <x:c r="AH12" s="43" t="str"/>
+      <x:c r="AI12" s="43" t="str"/>
+      <x:c r="AJ12" s="43" t="str"/>
+      <x:c r="AK12" s="43" t="str"/>
+      <x:c r="AL12" s="43" t="str"/>
+      <x:c r="AM12" s="43" t="str"/>
       <x:c r="AN12" s="32" t="str"/>
-      <x:c r="AO12" s="32" t="str"/>
-      <x:c r="AP12" s="32" t="str"/>
+      <x:c r="AO12" s="43" t="str"/>
+      <x:c r="AP12" s="43" t="str"/>
       <x:c r="AQ12" s="32" t="str"/>
-      <x:c r="AR12" s="32" t="str"/>
-      <x:c r="AS12" s="32" t="str"/>
+      <x:c r="AR12" s="43" t="str"/>
+      <x:c r="AS12" s="43" t="str"/>
       <x:c r="AT12" s="32" t="str"/>
       <x:c r="AU12" s="32" t="str"/>
       <x:c r="AV12" s="32" t="str"/>
-      <x:c r="AW12" s="33" t="str"/>
+      <x:c r="AW12" s="44" t="str"/>
       <x:c r="AX12" s="33" t="str"/>
       <x:c r="AY12" s="33" t="str"/>
       <x:c r="AZ12" s="33" t="str"/>
-      <x:c r="BA12" s="33" t="str">
+      <x:c r="BA12" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB12" s="33" t="str">
+      <x:c r="BB12" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC12" s="33" t="str">
+      <x:c r="BC12" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD12" s="33" t="str"/>
@@ -1595,58 +1606,58 @@
       <x:c r="E13" s="32" t="str"/>
       <x:c r="F13" s="32" t="str"/>
       <x:c r="G13" s="32" t="str"/>
-      <x:c r="H13" s="32" t="str"/>
-      <x:c r="I13" s="32" t="str"/>
-      <x:c r="J13" s="32" t="str"/>
-      <x:c r="K13" s="32" t="str"/>
-      <x:c r="L13" s="32" t="str"/>
-      <x:c r="M13" s="32" t="str"/>
-      <x:c r="N13" s="32" t="str"/>
-      <x:c r="O13" s="32" t="str"/>
-      <x:c r="P13" s="32" t="str"/>
-      <x:c r="Q13" s="32" t="str"/>
-      <x:c r="R13" s="32" t="str"/>
-      <x:c r="S13" s="32" t="str"/>
-      <x:c r="T13" s="32" t="str"/>
-      <x:c r="U13" s="32" t="str"/>
-      <x:c r="V13" s="32" t="str"/>
-      <x:c r="W13" s="32" t="str"/>
-      <x:c r="X13" s="32" t="str"/>
-      <x:c r="Y13" s="32" t="str"/>
-      <x:c r="Z13" s="32" t="str"/>
-      <x:c r="AA13" s="32" t="str"/>
-      <x:c r="AB13" s="32" t="str"/>
-      <x:c r="AC13" s="32" t="str"/>
-      <x:c r="AD13" s="32" t="str"/>
-      <x:c r="AE13" s="32" t="str"/>
-      <x:c r="AF13" s="32" t="str"/>
-      <x:c r="AG13" s="32" t="str"/>
-      <x:c r="AH13" s="32" t="str"/>
-      <x:c r="AI13" s="32" t="str"/>
-      <x:c r="AJ13" s="32" t="str"/>
-      <x:c r="AK13" s="32" t="str"/>
-      <x:c r="AL13" s="32" t="str"/>
-      <x:c r="AM13" s="32" t="str"/>
+      <x:c r="H13" s="43" t="str"/>
+      <x:c r="I13" s="43" t="str"/>
+      <x:c r="J13" s="43" t="str"/>
+      <x:c r="K13" s="43" t="str"/>
+      <x:c r="L13" s="43" t="str"/>
+      <x:c r="M13" s="43" t="str"/>
+      <x:c r="N13" s="43" t="str"/>
+      <x:c r="O13" s="43" t="str"/>
+      <x:c r="P13" s="43" t="str"/>
+      <x:c r="Q13" s="43" t="str"/>
+      <x:c r="R13" s="43" t="str"/>
+      <x:c r="S13" s="43" t="str"/>
+      <x:c r="T13" s="43" t="str"/>
+      <x:c r="U13" s="43" t="str"/>
+      <x:c r="V13" s="43" t="str"/>
+      <x:c r="W13" s="43" t="str"/>
+      <x:c r="X13" s="43" t="str"/>
+      <x:c r="Y13" s="43" t="str"/>
+      <x:c r="Z13" s="43" t="str"/>
+      <x:c r="AA13" s="43" t="str"/>
+      <x:c r="AB13" s="43" t="str"/>
+      <x:c r="AC13" s="43" t="str"/>
+      <x:c r="AD13" s="43" t="str"/>
+      <x:c r="AE13" s="43" t="str"/>
+      <x:c r="AF13" s="43" t="str"/>
+      <x:c r="AG13" s="43" t="str"/>
+      <x:c r="AH13" s="43" t="str"/>
+      <x:c r="AI13" s="43" t="str"/>
+      <x:c r="AJ13" s="43" t="str"/>
+      <x:c r="AK13" s="43" t="str"/>
+      <x:c r="AL13" s="43" t="str"/>
+      <x:c r="AM13" s="43" t="str"/>
       <x:c r="AN13" s="32" t="str"/>
-      <x:c r="AO13" s="32" t="str"/>
-      <x:c r="AP13" s="32" t="str"/>
+      <x:c r="AO13" s="43" t="str"/>
+      <x:c r="AP13" s="43" t="str"/>
       <x:c r="AQ13" s="32" t="str"/>
-      <x:c r="AR13" s="32" t="str"/>
-      <x:c r="AS13" s="32" t="str"/>
+      <x:c r="AR13" s="43" t="str"/>
+      <x:c r="AS13" s="43" t="str"/>
       <x:c r="AT13" s="32" t="str"/>
       <x:c r="AU13" s="32" t="str"/>
       <x:c r="AV13" s="32" t="str"/>
-      <x:c r="AW13" s="33" t="str"/>
+      <x:c r="AW13" s="44" t="str"/>
       <x:c r="AX13" s="33" t="str"/>
       <x:c r="AY13" s="33" t="str"/>
       <x:c r="AZ13" s="33" t="str"/>
-      <x:c r="BA13" s="33" t="str">
+      <x:c r="BA13" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB13" s="33" t="str">
+      <x:c r="BB13" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC13" s="33" t="str">
+      <x:c r="BC13" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD13" s="33" t="str"/>
@@ -1661,58 +1672,58 @@
       <x:c r="E14" s="32" t="str"/>
       <x:c r="F14" s="32" t="str"/>
       <x:c r="G14" s="32" t="str"/>
-      <x:c r="H14" s="32" t="str"/>
-      <x:c r="I14" s="32" t="str"/>
-      <x:c r="J14" s="32" t="str"/>
-      <x:c r="K14" s="32" t="str"/>
-      <x:c r="L14" s="32" t="str"/>
-      <x:c r="M14" s="32" t="str"/>
-      <x:c r="N14" s="32" t="str"/>
-      <x:c r="O14" s="32" t="str"/>
-      <x:c r="P14" s="32" t="str"/>
-      <x:c r="Q14" s="32" t="str"/>
-      <x:c r="R14" s="32" t="str"/>
-      <x:c r="S14" s="32" t="str"/>
-      <x:c r="T14" s="32" t="str"/>
-      <x:c r="U14" s="32" t="str"/>
-      <x:c r="V14" s="32" t="str"/>
-      <x:c r="W14" s="32" t="str"/>
-      <x:c r="X14" s="32" t="str"/>
-      <x:c r="Y14" s="32" t="str"/>
-      <x:c r="Z14" s="32" t="str"/>
-      <x:c r="AA14" s="32" t="str"/>
-      <x:c r="AB14" s="32" t="str"/>
-      <x:c r="AC14" s="32" t="str"/>
-      <x:c r="AD14" s="32" t="str"/>
-      <x:c r="AE14" s="32" t="str"/>
-      <x:c r="AF14" s="32" t="str"/>
-      <x:c r="AG14" s="32" t="str"/>
-      <x:c r="AH14" s="32" t="str"/>
-      <x:c r="AI14" s="32" t="str"/>
-      <x:c r="AJ14" s="32" t="str"/>
-      <x:c r="AK14" s="32" t="str"/>
-      <x:c r="AL14" s="32" t="str"/>
-      <x:c r="AM14" s="32" t="str"/>
+      <x:c r="H14" s="43" t="str"/>
+      <x:c r="I14" s="43" t="str"/>
+      <x:c r="J14" s="43" t="str"/>
+      <x:c r="K14" s="43" t="str"/>
+      <x:c r="L14" s="43" t="str"/>
+      <x:c r="M14" s="43" t="str"/>
+      <x:c r="N14" s="43" t="str"/>
+      <x:c r="O14" s="43" t="str"/>
+      <x:c r="P14" s="43" t="str"/>
+      <x:c r="Q14" s="43" t="str"/>
+      <x:c r="R14" s="43" t="str"/>
+      <x:c r="S14" s="43" t="str"/>
+      <x:c r="T14" s="43" t="str"/>
+      <x:c r="U14" s="43" t="str"/>
+      <x:c r="V14" s="43" t="str"/>
+      <x:c r="W14" s="43" t="str"/>
+      <x:c r="X14" s="43" t="str"/>
+      <x:c r="Y14" s="43" t="str"/>
+      <x:c r="Z14" s="43" t="str"/>
+      <x:c r="AA14" s="43" t="str"/>
+      <x:c r="AB14" s="43" t="str"/>
+      <x:c r="AC14" s="43" t="str"/>
+      <x:c r="AD14" s="43" t="str"/>
+      <x:c r="AE14" s="43" t="str"/>
+      <x:c r="AF14" s="43" t="str"/>
+      <x:c r="AG14" s="43" t="str"/>
+      <x:c r="AH14" s="43" t="str"/>
+      <x:c r="AI14" s="43" t="str"/>
+      <x:c r="AJ14" s="43" t="str"/>
+      <x:c r="AK14" s="43" t="str"/>
+      <x:c r="AL14" s="43" t="str"/>
+      <x:c r="AM14" s="43" t="str"/>
       <x:c r="AN14" s="32" t="str"/>
-      <x:c r="AO14" s="32" t="str"/>
-      <x:c r="AP14" s="32" t="str"/>
+      <x:c r="AO14" s="43" t="str"/>
+      <x:c r="AP14" s="43" t="str"/>
       <x:c r="AQ14" s="32" t="str"/>
-      <x:c r="AR14" s="32" t="str"/>
-      <x:c r="AS14" s="32" t="str"/>
+      <x:c r="AR14" s="43" t="str"/>
+      <x:c r="AS14" s="43" t="str"/>
       <x:c r="AT14" s="32" t="str"/>
       <x:c r="AU14" s="32" t="str"/>
       <x:c r="AV14" s="32" t="str"/>
-      <x:c r="AW14" s="33" t="str"/>
+      <x:c r="AW14" s="44" t="str"/>
       <x:c r="AX14" s="33" t="str"/>
       <x:c r="AY14" s="33" t="str"/>
       <x:c r="AZ14" s="33" t="str"/>
-      <x:c r="BA14" s="33" t="str">
+      <x:c r="BA14" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB14" s="33" t="str">
+      <x:c r="BB14" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC14" s="33" t="str">
+      <x:c r="BC14" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD14" s="33" t="str"/>
@@ -1727,58 +1738,58 @@
       <x:c r="E15" s="32" t="str"/>
       <x:c r="F15" s="32" t="str"/>
       <x:c r="G15" s="32" t="str"/>
-      <x:c r="H15" s="32" t="str"/>
-      <x:c r="I15" s="32" t="str"/>
-      <x:c r="J15" s="32" t="str"/>
-      <x:c r="K15" s="32" t="str"/>
-      <x:c r="L15" s="32" t="str"/>
-      <x:c r="M15" s="32" t="str"/>
-      <x:c r="N15" s="32" t="str"/>
-      <x:c r="O15" s="32" t="str"/>
-      <x:c r="P15" s="32" t="str"/>
-      <x:c r="Q15" s="32" t="str"/>
-      <x:c r="R15" s="32" t="str"/>
-      <x:c r="S15" s="32" t="str"/>
-      <x:c r="T15" s="32" t="str"/>
-      <x:c r="U15" s="32" t="str"/>
-      <x:c r="V15" s="32" t="str"/>
-      <x:c r="W15" s="32" t="str"/>
-      <x:c r="X15" s="32" t="str"/>
-      <x:c r="Y15" s="32" t="str"/>
-      <x:c r="Z15" s="32" t="str"/>
-      <x:c r="AA15" s="32" t="str"/>
-      <x:c r="AB15" s="32" t="str"/>
-      <x:c r="AC15" s="32" t="str"/>
-      <x:c r="AD15" s="32" t="str"/>
-      <x:c r="AE15" s="32" t="str"/>
-      <x:c r="AF15" s="32" t="str"/>
-      <x:c r="AG15" s="32" t="str"/>
-      <x:c r="AH15" s="32" t="str"/>
-      <x:c r="AI15" s="32" t="str"/>
-      <x:c r="AJ15" s="32" t="str"/>
-      <x:c r="AK15" s="32" t="str"/>
-      <x:c r="AL15" s="32" t="str"/>
-      <x:c r="AM15" s="32" t="str"/>
+      <x:c r="H15" s="43" t="str"/>
+      <x:c r="I15" s="43" t="str"/>
+      <x:c r="J15" s="43" t="str"/>
+      <x:c r="K15" s="43" t="str"/>
+      <x:c r="L15" s="43" t="str"/>
+      <x:c r="M15" s="43" t="str"/>
+      <x:c r="N15" s="43" t="str"/>
+      <x:c r="O15" s="43" t="str"/>
+      <x:c r="P15" s="43" t="str"/>
+      <x:c r="Q15" s="43" t="str"/>
+      <x:c r="R15" s="43" t="str"/>
+      <x:c r="S15" s="43" t="str"/>
+      <x:c r="T15" s="43" t="str"/>
+      <x:c r="U15" s="43" t="str"/>
+      <x:c r="V15" s="43" t="str"/>
+      <x:c r="W15" s="43" t="str"/>
+      <x:c r="X15" s="43" t="str"/>
+      <x:c r="Y15" s="43" t="str"/>
+      <x:c r="Z15" s="43" t="str"/>
+      <x:c r="AA15" s="43" t="str"/>
+      <x:c r="AB15" s="43" t="str"/>
+      <x:c r="AC15" s="43" t="str"/>
+      <x:c r="AD15" s="43" t="str"/>
+      <x:c r="AE15" s="43" t="str"/>
+      <x:c r="AF15" s="43" t="str"/>
+      <x:c r="AG15" s="43" t="str"/>
+      <x:c r="AH15" s="43" t="str"/>
+      <x:c r="AI15" s="43" t="str"/>
+      <x:c r="AJ15" s="43" t="str"/>
+      <x:c r="AK15" s="43" t="str"/>
+      <x:c r="AL15" s="43" t="str"/>
+      <x:c r="AM15" s="43" t="str"/>
       <x:c r="AN15" s="32" t="str"/>
-      <x:c r="AO15" s="32" t="str"/>
-      <x:c r="AP15" s="32" t="str"/>
+      <x:c r="AO15" s="43" t="str"/>
+      <x:c r="AP15" s="43" t="str"/>
       <x:c r="AQ15" s="32" t="str"/>
-      <x:c r="AR15" s="32" t="str"/>
-      <x:c r="AS15" s="32" t="str"/>
+      <x:c r="AR15" s="43" t="str"/>
+      <x:c r="AS15" s="43" t="str"/>
       <x:c r="AT15" s="32" t="str"/>
       <x:c r="AU15" s="32" t="str"/>
       <x:c r="AV15" s="32" t="str"/>
-      <x:c r="AW15" s="33" t="str"/>
+      <x:c r="AW15" s="44" t="str"/>
       <x:c r="AX15" s="33" t="str"/>
       <x:c r="AY15" s="33" t="str"/>
       <x:c r="AZ15" s="33" t="str"/>
-      <x:c r="BA15" s="33" t="str">
+      <x:c r="BA15" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB15" s="33" t="str">
+      <x:c r="BB15" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC15" s="33" t="str">
+      <x:c r="BC15" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD15" s="33" t="str"/>
@@ -1793,58 +1804,58 @@
       <x:c r="E16" s="32" t="str"/>
       <x:c r="F16" s="32" t="str"/>
       <x:c r="G16" s="32" t="str"/>
-      <x:c r="H16" s="32" t="str"/>
-      <x:c r="I16" s="32" t="str"/>
-      <x:c r="J16" s="32" t="str"/>
-      <x:c r="K16" s="32" t="str"/>
-      <x:c r="L16" s="32" t="str"/>
-      <x:c r="M16" s="32" t="str"/>
-      <x:c r="N16" s="32" t="str"/>
-      <x:c r="O16" s="32" t="str"/>
-      <x:c r="P16" s="32" t="str"/>
-      <x:c r="Q16" s="32" t="str"/>
-      <x:c r="R16" s="32" t="str"/>
-      <x:c r="S16" s="32" t="str"/>
-      <x:c r="T16" s="32" t="str"/>
-      <x:c r="U16" s="32" t="str"/>
-      <x:c r="V16" s="32" t="str"/>
-      <x:c r="W16" s="32" t="str"/>
-      <x:c r="X16" s="32" t="str"/>
-      <x:c r="Y16" s="32" t="str"/>
-      <x:c r="Z16" s="32" t="str"/>
-      <x:c r="AA16" s="32" t="str"/>
-      <x:c r="AB16" s="32" t="str"/>
-      <x:c r="AC16" s="32" t="str"/>
-      <x:c r="AD16" s="32" t="str"/>
-      <x:c r="AE16" s="32" t="str"/>
-      <x:c r="AF16" s="32" t="str"/>
-      <x:c r="AG16" s="32" t="str"/>
-      <x:c r="AH16" s="32" t="str"/>
-      <x:c r="AI16" s="32" t="str"/>
-      <x:c r="AJ16" s="32" t="str"/>
-      <x:c r="AK16" s="32" t="str"/>
-      <x:c r="AL16" s="32" t="str"/>
-      <x:c r="AM16" s="32" t="str"/>
+      <x:c r="H16" s="43" t="str"/>
+      <x:c r="I16" s="43" t="str"/>
+      <x:c r="J16" s="43" t="str"/>
+      <x:c r="K16" s="43" t="str"/>
+      <x:c r="L16" s="43" t="str"/>
+      <x:c r="M16" s="43" t="str"/>
+      <x:c r="N16" s="43" t="str"/>
+      <x:c r="O16" s="43" t="str"/>
+      <x:c r="P16" s="43" t="str"/>
+      <x:c r="Q16" s="43" t="str"/>
+      <x:c r="R16" s="43" t="str"/>
+      <x:c r="S16" s="43" t="str"/>
+      <x:c r="T16" s="43" t="str"/>
+      <x:c r="U16" s="43" t="str"/>
+      <x:c r="V16" s="43" t="str"/>
+      <x:c r="W16" s="43" t="str"/>
+      <x:c r="X16" s="43" t="str"/>
+      <x:c r="Y16" s="43" t="str"/>
+      <x:c r="Z16" s="43" t="str"/>
+      <x:c r="AA16" s="43" t="str"/>
+      <x:c r="AB16" s="43" t="str"/>
+      <x:c r="AC16" s="43" t="str"/>
+      <x:c r="AD16" s="43" t="str"/>
+      <x:c r="AE16" s="43" t="str"/>
+      <x:c r="AF16" s="43" t="str"/>
+      <x:c r="AG16" s="43" t="str"/>
+      <x:c r="AH16" s="43" t="str"/>
+      <x:c r="AI16" s="43" t="str"/>
+      <x:c r="AJ16" s="43" t="str"/>
+      <x:c r="AK16" s="43" t="str"/>
+      <x:c r="AL16" s="43" t="str"/>
+      <x:c r="AM16" s="43" t="str"/>
       <x:c r="AN16" s="32" t="str"/>
-      <x:c r="AO16" s="32" t="str"/>
-      <x:c r="AP16" s="32" t="str"/>
+      <x:c r="AO16" s="43" t="str"/>
+      <x:c r="AP16" s="43" t="str"/>
       <x:c r="AQ16" s="32" t="str"/>
-      <x:c r="AR16" s="32" t="str"/>
-      <x:c r="AS16" s="32" t="str"/>
+      <x:c r="AR16" s="43" t="str"/>
+      <x:c r="AS16" s="43" t="str"/>
       <x:c r="AT16" s="32" t="str"/>
       <x:c r="AU16" s="32" t="str"/>
       <x:c r="AV16" s="32" t="str"/>
-      <x:c r="AW16" s="33" t="str"/>
+      <x:c r="AW16" s="44" t="str"/>
       <x:c r="AX16" s="33" t="str"/>
       <x:c r="AY16" s="33" t="str"/>
       <x:c r="AZ16" s="33" t="str"/>
-      <x:c r="BA16" s="33" t="str">
+      <x:c r="BA16" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB16" s="33" t="str">
+      <x:c r="BB16" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC16" s="33" t="str">
+      <x:c r="BC16" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD16" s="33" t="str"/>
@@ -1859,58 +1870,58 @@
       <x:c r="E17" s="32" t="str"/>
       <x:c r="F17" s="32" t="str"/>
       <x:c r="G17" s="32" t="str"/>
-      <x:c r="H17" s="32" t="str"/>
-      <x:c r="I17" s="32" t="str"/>
-      <x:c r="J17" s="32" t="str"/>
-      <x:c r="K17" s="32" t="str"/>
-      <x:c r="L17" s="32" t="str"/>
-      <x:c r="M17" s="32" t="str"/>
-      <x:c r="N17" s="32" t="str"/>
-      <x:c r="O17" s="32" t="str"/>
-      <x:c r="P17" s="32" t="str"/>
-      <x:c r="Q17" s="32" t="str"/>
-      <x:c r="R17" s="32" t="str"/>
-      <x:c r="S17" s="32" t="str"/>
-      <x:c r="T17" s="32" t="str"/>
-      <x:c r="U17" s="32" t="str"/>
-      <x:c r="V17" s="32" t="str"/>
-      <x:c r="W17" s="32" t="str"/>
-      <x:c r="X17" s="32" t="str"/>
-      <x:c r="Y17" s="32" t="str"/>
-      <x:c r="Z17" s="32" t="str"/>
-      <x:c r="AA17" s="32" t="str"/>
-      <x:c r="AB17" s="32" t="str"/>
-      <x:c r="AC17" s="32" t="str"/>
-      <x:c r="AD17" s="32" t="str"/>
-      <x:c r="AE17" s="32" t="str"/>
-      <x:c r="AF17" s="32" t="str"/>
-      <x:c r="AG17" s="32" t="str"/>
-      <x:c r="AH17" s="32" t="str"/>
-      <x:c r="AI17" s="32" t="str"/>
-      <x:c r="AJ17" s="32" t="str"/>
-      <x:c r="AK17" s="32" t="str"/>
-      <x:c r="AL17" s="32" t="str"/>
-      <x:c r="AM17" s="32" t="str"/>
+      <x:c r="H17" s="43" t="str"/>
+      <x:c r="I17" s="43" t="str"/>
+      <x:c r="J17" s="43" t="str"/>
+      <x:c r="K17" s="43" t="str"/>
+      <x:c r="L17" s="43" t="str"/>
+      <x:c r="M17" s="43" t="str"/>
+      <x:c r="N17" s="43" t="str"/>
+      <x:c r="O17" s="43" t="str"/>
+      <x:c r="P17" s="43" t="str"/>
+      <x:c r="Q17" s="43" t="str"/>
+      <x:c r="R17" s="43" t="str"/>
+      <x:c r="S17" s="43" t="str"/>
+      <x:c r="T17" s="43" t="str"/>
+      <x:c r="U17" s="43" t="str"/>
+      <x:c r="V17" s="43" t="str"/>
+      <x:c r="W17" s="43" t="str"/>
+      <x:c r="X17" s="43" t="str"/>
+      <x:c r="Y17" s="43" t="str"/>
+      <x:c r="Z17" s="43" t="str"/>
+      <x:c r="AA17" s="43" t="str"/>
+      <x:c r="AB17" s="43" t="str"/>
+      <x:c r="AC17" s="43" t="str"/>
+      <x:c r="AD17" s="43" t="str"/>
+      <x:c r="AE17" s="43" t="str"/>
+      <x:c r="AF17" s="43" t="str"/>
+      <x:c r="AG17" s="43" t="str"/>
+      <x:c r="AH17" s="43" t="str"/>
+      <x:c r="AI17" s="43" t="str"/>
+      <x:c r="AJ17" s="43" t="str"/>
+      <x:c r="AK17" s="43" t="str"/>
+      <x:c r="AL17" s="43" t="str"/>
+      <x:c r="AM17" s="43" t="str"/>
       <x:c r="AN17" s="32" t="str"/>
-      <x:c r="AO17" s="32" t="str"/>
-      <x:c r="AP17" s="32" t="str"/>
+      <x:c r="AO17" s="43" t="str"/>
+      <x:c r="AP17" s="43" t="str"/>
       <x:c r="AQ17" s="32" t="str"/>
-      <x:c r="AR17" s="32" t="str"/>
-      <x:c r="AS17" s="32" t="str"/>
+      <x:c r="AR17" s="43" t="str"/>
+      <x:c r="AS17" s="43" t="str"/>
       <x:c r="AT17" s="32" t="str"/>
       <x:c r="AU17" s="32" t="str"/>
       <x:c r="AV17" s="32" t="str"/>
-      <x:c r="AW17" s="33" t="str"/>
+      <x:c r="AW17" s="44" t="str"/>
       <x:c r="AX17" s="33" t="str"/>
       <x:c r="AY17" s="33" t="str"/>
       <x:c r="AZ17" s="33" t="str"/>
-      <x:c r="BA17" s="33" t="str">
+      <x:c r="BA17" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB17" s="33" t="str">
+      <x:c r="BB17" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC17" s="33" t="str">
+      <x:c r="BC17" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD17" s="33" t="str"/>
@@ -1925,58 +1936,58 @@
       <x:c r="E18" s="32" t="str"/>
       <x:c r="F18" s="32" t="str"/>
       <x:c r="G18" s="32" t="str"/>
-      <x:c r="H18" s="32" t="str"/>
-      <x:c r="I18" s="32" t="str"/>
-      <x:c r="J18" s="32" t="str"/>
-      <x:c r="K18" s="32" t="str"/>
-      <x:c r="L18" s="32" t="str"/>
-      <x:c r="M18" s="32" t="str"/>
-      <x:c r="N18" s="32" t="str"/>
-      <x:c r="O18" s="32" t="str"/>
-      <x:c r="P18" s="32" t="str"/>
-      <x:c r="Q18" s="32" t="str"/>
-      <x:c r="R18" s="32" t="str"/>
-      <x:c r="S18" s="32" t="str"/>
-      <x:c r="T18" s="32" t="str"/>
-      <x:c r="U18" s="32" t="str"/>
-      <x:c r="V18" s="32" t="str"/>
-      <x:c r="W18" s="32" t="str"/>
-      <x:c r="X18" s="32" t="str"/>
-      <x:c r="Y18" s="32" t="str"/>
-      <x:c r="Z18" s="32" t="str"/>
-      <x:c r="AA18" s="32" t="str"/>
-      <x:c r="AB18" s="32" t="str"/>
-      <x:c r="AC18" s="32" t="str"/>
-      <x:c r="AD18" s="32" t="str"/>
-      <x:c r="AE18" s="32" t="str"/>
-      <x:c r="AF18" s="32" t="str"/>
-      <x:c r="AG18" s="32" t="str"/>
-      <x:c r="AH18" s="32" t="str"/>
-      <x:c r="AI18" s="32" t="str"/>
-      <x:c r="AJ18" s="32" t="str"/>
-      <x:c r="AK18" s="32" t="str"/>
-      <x:c r="AL18" s="32" t="str"/>
-      <x:c r="AM18" s="32" t="str"/>
+      <x:c r="H18" s="43" t="str"/>
+      <x:c r="I18" s="43" t="str"/>
+      <x:c r="J18" s="43" t="str"/>
+      <x:c r="K18" s="43" t="str"/>
+      <x:c r="L18" s="43" t="str"/>
+      <x:c r="M18" s="43" t="str"/>
+      <x:c r="N18" s="43" t="str"/>
+      <x:c r="O18" s="43" t="str"/>
+      <x:c r="P18" s="43" t="str"/>
+      <x:c r="Q18" s="43" t="str"/>
+      <x:c r="R18" s="43" t="str"/>
+      <x:c r="S18" s="43" t="str"/>
+      <x:c r="T18" s="43" t="str"/>
+      <x:c r="U18" s="43" t="str"/>
+      <x:c r="V18" s="43" t="str"/>
+      <x:c r="W18" s="43" t="str"/>
+      <x:c r="X18" s="43" t="str"/>
+      <x:c r="Y18" s="43" t="str"/>
+      <x:c r="Z18" s="43" t="str"/>
+      <x:c r="AA18" s="43" t="str"/>
+      <x:c r="AB18" s="43" t="str"/>
+      <x:c r="AC18" s="43" t="str"/>
+      <x:c r="AD18" s="43" t="str"/>
+      <x:c r="AE18" s="43" t="str"/>
+      <x:c r="AF18" s="43" t="str"/>
+      <x:c r="AG18" s="43" t="str"/>
+      <x:c r="AH18" s="43" t="str"/>
+      <x:c r="AI18" s="43" t="str"/>
+      <x:c r="AJ18" s="43" t="str"/>
+      <x:c r="AK18" s="43" t="str"/>
+      <x:c r="AL18" s="43" t="str"/>
+      <x:c r="AM18" s="43" t="str"/>
       <x:c r="AN18" s="32" t="str"/>
-      <x:c r="AO18" s="32" t="str"/>
-      <x:c r="AP18" s="32" t="str"/>
+      <x:c r="AO18" s="43" t="str"/>
+      <x:c r="AP18" s="43" t="str"/>
       <x:c r="AQ18" s="32" t="str"/>
-      <x:c r="AR18" s="32" t="str"/>
-      <x:c r="AS18" s="32" t="str"/>
+      <x:c r="AR18" s="43" t="str"/>
+      <x:c r="AS18" s="43" t="str"/>
       <x:c r="AT18" s="32" t="str"/>
       <x:c r="AU18" s="32" t="str"/>
       <x:c r="AV18" s="32" t="str"/>
-      <x:c r="AW18" s="33" t="str"/>
+      <x:c r="AW18" s="44" t="str"/>
       <x:c r="AX18" s="33" t="str"/>
       <x:c r="AY18" s="33" t="str"/>
       <x:c r="AZ18" s="33" t="str"/>
-      <x:c r="BA18" s="33" t="str">
+      <x:c r="BA18" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB18" s="33" t="str">
+      <x:c r="BB18" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC18" s="33" t="str">
+      <x:c r="BC18" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD18" s="33" t="str"/>
@@ -1991,58 +2002,58 @@
       <x:c r="E19" s="32" t="str"/>
       <x:c r="F19" s="32" t="str"/>
       <x:c r="G19" s="32" t="str"/>
-      <x:c r="H19" s="32" t="str"/>
-      <x:c r="I19" s="32" t="str"/>
-      <x:c r="J19" s="32" t="str"/>
-      <x:c r="K19" s="32" t="str"/>
-      <x:c r="L19" s="32" t="str"/>
-      <x:c r="M19" s="32" t="str"/>
-      <x:c r="N19" s="32" t="str"/>
-      <x:c r="O19" s="32" t="str"/>
-      <x:c r="P19" s="32" t="str"/>
-      <x:c r="Q19" s="32" t="str"/>
-      <x:c r="R19" s="32" t="str"/>
-      <x:c r="S19" s="32" t="str"/>
-      <x:c r="T19" s="32" t="str"/>
-      <x:c r="U19" s="32" t="str"/>
-      <x:c r="V19" s="32" t="str"/>
-      <x:c r="W19" s="32" t="str"/>
-      <x:c r="X19" s="32" t="str"/>
-      <x:c r="Y19" s="32" t="str"/>
-      <x:c r="Z19" s="32" t="str"/>
-      <x:c r="AA19" s="32" t="str"/>
-      <x:c r="AB19" s="32" t="str"/>
-      <x:c r="AC19" s="32" t="str"/>
-      <x:c r="AD19" s="32" t="str"/>
-      <x:c r="AE19" s="32" t="str"/>
-      <x:c r="AF19" s="32" t="str"/>
-      <x:c r="AG19" s="32" t="str"/>
-      <x:c r="AH19" s="32" t="str"/>
-      <x:c r="AI19" s="32" t="str"/>
-      <x:c r="AJ19" s="32" t="str"/>
-      <x:c r="AK19" s="32" t="str"/>
-      <x:c r="AL19" s="32" t="str"/>
-      <x:c r="AM19" s="32" t="str"/>
+      <x:c r="H19" s="43" t="str"/>
+      <x:c r="I19" s="43" t="str"/>
+      <x:c r="J19" s="43" t="str"/>
+      <x:c r="K19" s="43" t="str"/>
+      <x:c r="L19" s="43" t="str"/>
+      <x:c r="M19" s="43" t="str"/>
+      <x:c r="N19" s="43" t="str"/>
+      <x:c r="O19" s="43" t="str"/>
+      <x:c r="P19" s="43" t="str"/>
+      <x:c r="Q19" s="43" t="str"/>
+      <x:c r="R19" s="43" t="str"/>
+      <x:c r="S19" s="43" t="str"/>
+      <x:c r="T19" s="43" t="str"/>
+      <x:c r="U19" s="43" t="str"/>
+      <x:c r="V19" s="43" t="str"/>
+      <x:c r="W19" s="43" t="str"/>
+      <x:c r="X19" s="43" t="str"/>
+      <x:c r="Y19" s="43" t="str"/>
+      <x:c r="Z19" s="43" t="str"/>
+      <x:c r="AA19" s="43" t="str"/>
+      <x:c r="AB19" s="43" t="str"/>
+      <x:c r="AC19" s="43" t="str"/>
+      <x:c r="AD19" s="43" t="str"/>
+      <x:c r="AE19" s="43" t="str"/>
+      <x:c r="AF19" s="43" t="str"/>
+      <x:c r="AG19" s="43" t="str"/>
+      <x:c r="AH19" s="43" t="str"/>
+      <x:c r="AI19" s="43" t="str"/>
+      <x:c r="AJ19" s="43" t="str"/>
+      <x:c r="AK19" s="43" t="str"/>
+      <x:c r="AL19" s="43" t="str"/>
+      <x:c r="AM19" s="43" t="str"/>
       <x:c r="AN19" s="32" t="str"/>
-      <x:c r="AO19" s="32" t="str"/>
-      <x:c r="AP19" s="32" t="str"/>
+      <x:c r="AO19" s="43" t="str"/>
+      <x:c r="AP19" s="43" t="str"/>
       <x:c r="AQ19" s="32" t="str"/>
-      <x:c r="AR19" s="32" t="str"/>
-      <x:c r="AS19" s="32" t="str"/>
+      <x:c r="AR19" s="43" t="str"/>
+      <x:c r="AS19" s="43" t="str"/>
       <x:c r="AT19" s="32" t="str"/>
       <x:c r="AU19" s="32" t="str"/>
       <x:c r="AV19" s="32" t="str"/>
-      <x:c r="AW19" s="33" t="str"/>
+      <x:c r="AW19" s="44" t="str"/>
       <x:c r="AX19" s="33" t="str"/>
       <x:c r="AY19" s="33" t="str"/>
       <x:c r="AZ19" s="33" t="str"/>
-      <x:c r="BA19" s="33" t="str">
+      <x:c r="BA19" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB19" s="33" t="str">
+      <x:c r="BB19" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC19" s="33" t="str">
+      <x:c r="BC19" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD19" s="33" t="str"/>
@@ -2057,58 +2068,58 @@
       <x:c r="E20" s="32" t="str"/>
       <x:c r="F20" s="32" t="str"/>
       <x:c r="G20" s="32" t="str"/>
-      <x:c r="H20" s="32" t="str"/>
-      <x:c r="I20" s="32" t="str"/>
-      <x:c r="J20" s="32" t="str"/>
-      <x:c r="K20" s="32" t="str"/>
-      <x:c r="L20" s="32" t="str"/>
-      <x:c r="M20" s="32" t="str"/>
-      <x:c r="N20" s="32" t="str"/>
-      <x:c r="O20" s="32" t="str"/>
-      <x:c r="P20" s="32" t="str"/>
-      <x:c r="Q20" s="32" t="str"/>
-      <x:c r="R20" s="32" t="str"/>
-      <x:c r="S20" s="32" t="str"/>
-      <x:c r="T20" s="32" t="str"/>
-      <x:c r="U20" s="32" t="str"/>
-      <x:c r="V20" s="32" t="str"/>
-      <x:c r="W20" s="32" t="str"/>
-      <x:c r="X20" s="32" t="str"/>
-      <x:c r="Y20" s="32" t="str"/>
-      <x:c r="Z20" s="32" t="str"/>
-      <x:c r="AA20" s="32" t="str"/>
-      <x:c r="AB20" s="32" t="str"/>
-      <x:c r="AC20" s="32" t="str"/>
-      <x:c r="AD20" s="32" t="str"/>
-      <x:c r="AE20" s="32" t="str"/>
-      <x:c r="AF20" s="32" t="str"/>
-      <x:c r="AG20" s="32" t="str"/>
-      <x:c r="AH20" s="32" t="str"/>
-      <x:c r="AI20" s="32" t="str"/>
-      <x:c r="AJ20" s="32" t="str"/>
-      <x:c r="AK20" s="32" t="str"/>
-      <x:c r="AL20" s="32" t="str"/>
-      <x:c r="AM20" s="32" t="str"/>
+      <x:c r="H20" s="43" t="str"/>
+      <x:c r="I20" s="43" t="str"/>
+      <x:c r="J20" s="43" t="str"/>
+      <x:c r="K20" s="43" t="str"/>
+      <x:c r="L20" s="43" t="str"/>
+      <x:c r="M20" s="43" t="str"/>
+      <x:c r="N20" s="43" t="str"/>
+      <x:c r="O20" s="43" t="str"/>
+      <x:c r="P20" s="43" t="str"/>
+      <x:c r="Q20" s="43" t="str"/>
+      <x:c r="R20" s="43" t="str"/>
+      <x:c r="S20" s="43" t="str"/>
+      <x:c r="T20" s="43" t="str"/>
+      <x:c r="U20" s="43" t="str"/>
+      <x:c r="V20" s="43" t="str"/>
+      <x:c r="W20" s="43" t="str"/>
+      <x:c r="X20" s="43" t="str"/>
+      <x:c r="Y20" s="43" t="str"/>
+      <x:c r="Z20" s="43" t="str"/>
+      <x:c r="AA20" s="43" t="str"/>
+      <x:c r="AB20" s="43" t="str"/>
+      <x:c r="AC20" s="43" t="str"/>
+      <x:c r="AD20" s="43" t="str"/>
+      <x:c r="AE20" s="43" t="str"/>
+      <x:c r="AF20" s="43" t="str"/>
+      <x:c r="AG20" s="43" t="str"/>
+      <x:c r="AH20" s="43" t="str"/>
+      <x:c r="AI20" s="43" t="str"/>
+      <x:c r="AJ20" s="43" t="str"/>
+      <x:c r="AK20" s="43" t="str"/>
+      <x:c r="AL20" s="43" t="str"/>
+      <x:c r="AM20" s="43" t="str"/>
       <x:c r="AN20" s="32" t="str"/>
-      <x:c r="AO20" s="32" t="str"/>
-      <x:c r="AP20" s="32" t="str"/>
+      <x:c r="AO20" s="43" t="str"/>
+      <x:c r="AP20" s="43" t="str"/>
       <x:c r="AQ20" s="32" t="str"/>
-      <x:c r="AR20" s="32" t="str"/>
-      <x:c r="AS20" s="32" t="str"/>
+      <x:c r="AR20" s="43" t="str"/>
+      <x:c r="AS20" s="43" t="str"/>
       <x:c r="AT20" s="32" t="str"/>
       <x:c r="AU20" s="32" t="str"/>
       <x:c r="AV20" s="32" t="str"/>
-      <x:c r="AW20" s="33" t="str"/>
+      <x:c r="AW20" s="44" t="str"/>
       <x:c r="AX20" s="33" t="str"/>
       <x:c r="AY20" s="33" t="str"/>
       <x:c r="AZ20" s="33" t="str"/>
-      <x:c r="BA20" s="33" t="str">
+      <x:c r="BA20" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB20" s="33" t="str">
+      <x:c r="BB20" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC20" s="33" t="str">
+      <x:c r="BC20" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD20" s="33" t="str"/>
@@ -2123,58 +2134,58 @@
       <x:c r="E21" s="32" t="str"/>
       <x:c r="F21" s="32" t="str"/>
       <x:c r="G21" s="32" t="str"/>
-      <x:c r="H21" s="32" t="str"/>
-      <x:c r="I21" s="32" t="str"/>
-      <x:c r="J21" s="32" t="str"/>
-      <x:c r="K21" s="32" t="str"/>
-      <x:c r="L21" s="32" t="str"/>
-      <x:c r="M21" s="32" t="str"/>
-      <x:c r="N21" s="32" t="str"/>
-      <x:c r="O21" s="32" t="str"/>
-      <x:c r="P21" s="32" t="str"/>
-      <x:c r="Q21" s="32" t="str"/>
-      <x:c r="R21" s="32" t="str"/>
-      <x:c r="S21" s="32" t="str"/>
-      <x:c r="T21" s="32" t="str"/>
-      <x:c r="U21" s="32" t="str"/>
-      <x:c r="V21" s="32" t="str"/>
-      <x:c r="W21" s="32" t="str"/>
-      <x:c r="X21" s="32" t="str"/>
-      <x:c r="Y21" s="32" t="str"/>
-      <x:c r="Z21" s="32" t="str"/>
-      <x:c r="AA21" s="32" t="str"/>
-      <x:c r="AB21" s="32" t="str"/>
-      <x:c r="AC21" s="32" t="str"/>
-      <x:c r="AD21" s="32" t="str"/>
-      <x:c r="AE21" s="32" t="str"/>
-      <x:c r="AF21" s="32" t="str"/>
-      <x:c r="AG21" s="32" t="str"/>
-      <x:c r="AH21" s="32" t="str"/>
-      <x:c r="AI21" s="32" t="str"/>
-      <x:c r="AJ21" s="32" t="str"/>
-      <x:c r="AK21" s="32" t="str"/>
-      <x:c r="AL21" s="32" t="str"/>
-      <x:c r="AM21" s="32" t="str"/>
+      <x:c r="H21" s="43" t="str"/>
+      <x:c r="I21" s="43" t="str"/>
+      <x:c r="J21" s="43" t="str"/>
+      <x:c r="K21" s="43" t="str"/>
+      <x:c r="L21" s="43" t="str"/>
+      <x:c r="M21" s="43" t="str"/>
+      <x:c r="N21" s="43" t="str"/>
+      <x:c r="O21" s="43" t="str"/>
+      <x:c r="P21" s="43" t="str"/>
+      <x:c r="Q21" s="43" t="str"/>
+      <x:c r="R21" s="43" t="str"/>
+      <x:c r="S21" s="43" t="str"/>
+      <x:c r="T21" s="43" t="str"/>
+      <x:c r="U21" s="43" t="str"/>
+      <x:c r="V21" s="43" t="str"/>
+      <x:c r="W21" s="43" t="str"/>
+      <x:c r="X21" s="43" t="str"/>
+      <x:c r="Y21" s="43" t="str"/>
+      <x:c r="Z21" s="43" t="str"/>
+      <x:c r="AA21" s="43" t="str"/>
+      <x:c r="AB21" s="43" t="str"/>
+      <x:c r="AC21" s="43" t="str"/>
+      <x:c r="AD21" s="43" t="str"/>
+      <x:c r="AE21" s="43" t="str"/>
+      <x:c r="AF21" s="43" t="str"/>
+      <x:c r="AG21" s="43" t="str"/>
+      <x:c r="AH21" s="43" t="str"/>
+      <x:c r="AI21" s="43" t="str"/>
+      <x:c r="AJ21" s="43" t="str"/>
+      <x:c r="AK21" s="43" t="str"/>
+      <x:c r="AL21" s="43" t="str"/>
+      <x:c r="AM21" s="43" t="str"/>
       <x:c r="AN21" s="32" t="str"/>
-      <x:c r="AO21" s="32" t="str"/>
-      <x:c r="AP21" s="32" t="str"/>
+      <x:c r="AO21" s="43" t="str"/>
+      <x:c r="AP21" s="43" t="str"/>
       <x:c r="AQ21" s="32" t="str"/>
-      <x:c r="AR21" s="32" t="str"/>
-      <x:c r="AS21" s="32" t="str"/>
+      <x:c r="AR21" s="43" t="str"/>
+      <x:c r="AS21" s="43" t="str"/>
       <x:c r="AT21" s="32" t="str"/>
       <x:c r="AU21" s="32" t="str"/>
       <x:c r="AV21" s="32" t="str"/>
-      <x:c r="AW21" s="33" t="str"/>
+      <x:c r="AW21" s="44" t="str"/>
       <x:c r="AX21" s="33" t="str"/>
       <x:c r="AY21" s="33" t="str"/>
       <x:c r="AZ21" s="33" t="str"/>
-      <x:c r="BA21" s="33" t="str">
+      <x:c r="BA21" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB21" s="33" t="str">
+      <x:c r="BB21" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC21" s="33" t="str">
+      <x:c r="BC21" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD21" s="33" t="str"/>
@@ -2189,58 +2200,58 @@
       <x:c r="E22" s="32" t="str"/>
       <x:c r="F22" s="32" t="str"/>
       <x:c r="G22" s="32" t="str"/>
-      <x:c r="H22" s="32" t="str"/>
-      <x:c r="I22" s="32" t="str"/>
-      <x:c r="J22" s="32" t="str"/>
-      <x:c r="K22" s="32" t="str"/>
-      <x:c r="L22" s="32" t="str"/>
-      <x:c r="M22" s="32" t="str"/>
-      <x:c r="N22" s="32" t="str"/>
-      <x:c r="O22" s="32" t="str"/>
-      <x:c r="P22" s="32" t="str"/>
-      <x:c r="Q22" s="32" t="str"/>
-      <x:c r="R22" s="32" t="str"/>
-      <x:c r="S22" s="32" t="str"/>
-      <x:c r="T22" s="32" t="str"/>
-      <x:c r="U22" s="32" t="str"/>
-      <x:c r="V22" s="32" t="str"/>
-      <x:c r="W22" s="32" t="str"/>
-      <x:c r="X22" s="32" t="str"/>
-      <x:c r="Y22" s="32" t="str"/>
-      <x:c r="Z22" s="32" t="str"/>
-      <x:c r="AA22" s="32" t="str"/>
-      <x:c r="AB22" s="32" t="str"/>
-      <x:c r="AC22" s="32" t="str"/>
-      <x:c r="AD22" s="32" t="str"/>
-      <x:c r="AE22" s="32" t="str"/>
-      <x:c r="AF22" s="32" t="str"/>
-      <x:c r="AG22" s="32" t="str"/>
-      <x:c r="AH22" s="32" t="str"/>
-      <x:c r="AI22" s="32" t="str"/>
-      <x:c r="AJ22" s="32" t="str"/>
-      <x:c r="AK22" s="32" t="str"/>
-      <x:c r="AL22" s="32" t="str"/>
-      <x:c r="AM22" s="32" t="str"/>
+      <x:c r="H22" s="43" t="str"/>
+      <x:c r="I22" s="43" t="str"/>
+      <x:c r="J22" s="43" t="str"/>
+      <x:c r="K22" s="43" t="str"/>
+      <x:c r="L22" s="43" t="str"/>
+      <x:c r="M22" s="43" t="str"/>
+      <x:c r="N22" s="43" t="str"/>
+      <x:c r="O22" s="43" t="str"/>
+      <x:c r="P22" s="43" t="str"/>
+      <x:c r="Q22" s="43" t="str"/>
+      <x:c r="R22" s="43" t="str"/>
+      <x:c r="S22" s="43" t="str"/>
+      <x:c r="T22" s="43" t="str"/>
+      <x:c r="U22" s="43" t="str"/>
+      <x:c r="V22" s="43" t="str"/>
+      <x:c r="W22" s="43" t="str"/>
+      <x:c r="X22" s="43" t="str"/>
+      <x:c r="Y22" s="43" t="str"/>
+      <x:c r="Z22" s="43" t="str"/>
+      <x:c r="AA22" s="43" t="str"/>
+      <x:c r="AB22" s="43" t="str"/>
+      <x:c r="AC22" s="43" t="str"/>
+      <x:c r="AD22" s="43" t="str"/>
+      <x:c r="AE22" s="43" t="str"/>
+      <x:c r="AF22" s="43" t="str"/>
+      <x:c r="AG22" s="43" t="str"/>
+      <x:c r="AH22" s="43" t="str"/>
+      <x:c r="AI22" s="43" t="str"/>
+      <x:c r="AJ22" s="43" t="str"/>
+      <x:c r="AK22" s="43" t="str"/>
+      <x:c r="AL22" s="43" t="str"/>
+      <x:c r="AM22" s="43" t="str"/>
       <x:c r="AN22" s="32" t="str"/>
-      <x:c r="AO22" s="32" t="str"/>
-      <x:c r="AP22" s="32" t="str"/>
+      <x:c r="AO22" s="43" t="str"/>
+      <x:c r="AP22" s="43" t="str"/>
       <x:c r="AQ22" s="32" t="str"/>
-      <x:c r="AR22" s="32" t="str"/>
-      <x:c r="AS22" s="32" t="str"/>
+      <x:c r="AR22" s="43" t="str"/>
+      <x:c r="AS22" s="43" t="str"/>
       <x:c r="AT22" s="32" t="str"/>
       <x:c r="AU22" s="32" t="str"/>
       <x:c r="AV22" s="32" t="str"/>
-      <x:c r="AW22" s="33" t="str"/>
+      <x:c r="AW22" s="44" t="str"/>
       <x:c r="AX22" s="33" t="str"/>
       <x:c r="AY22" s="33" t="str"/>
       <x:c r="AZ22" s="33" t="str"/>
-      <x:c r="BA22" s="33" t="str">
+      <x:c r="BA22" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB22" s="33" t="str">
+      <x:c r="BB22" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC22" s="33" t="str">
+      <x:c r="BC22" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD22" s="33" t="str"/>
@@ -2255,58 +2266,58 @@
       <x:c r="E23" s="32" t="str"/>
       <x:c r="F23" s="32" t="str"/>
       <x:c r="G23" s="32" t="str"/>
-      <x:c r="H23" s="32" t="str"/>
-      <x:c r="I23" s="32" t="str"/>
-      <x:c r="J23" s="32" t="str"/>
-      <x:c r="K23" s="32" t="str"/>
-      <x:c r="L23" s="32" t="str"/>
-      <x:c r="M23" s="32" t="str"/>
-      <x:c r="N23" s="32" t="str"/>
-      <x:c r="O23" s="32" t="str"/>
-      <x:c r="P23" s="32" t="str"/>
-      <x:c r="Q23" s="32" t="str"/>
-      <x:c r="R23" s="32" t="str"/>
-      <x:c r="S23" s="32" t="str"/>
-      <x:c r="T23" s="32" t="str"/>
-      <x:c r="U23" s="32" t="str"/>
-      <x:c r="V23" s="32" t="str"/>
-      <x:c r="W23" s="32" t="str"/>
-      <x:c r="X23" s="32" t="str"/>
-      <x:c r="Y23" s="32" t="str"/>
-      <x:c r="Z23" s="32" t="str"/>
-      <x:c r="AA23" s="32" t="str"/>
-      <x:c r="AB23" s="32" t="str"/>
-      <x:c r="AC23" s="32" t="str"/>
-      <x:c r="AD23" s="32" t="str"/>
-      <x:c r="AE23" s="32" t="str"/>
-      <x:c r="AF23" s="32" t="str"/>
-      <x:c r="AG23" s="32" t="str"/>
-      <x:c r="AH23" s="32" t="str"/>
-      <x:c r="AI23" s="32" t="str"/>
-      <x:c r="AJ23" s="32" t="str"/>
-      <x:c r="AK23" s="32" t="str"/>
-      <x:c r="AL23" s="32" t="str"/>
-      <x:c r="AM23" s="32" t="str"/>
+      <x:c r="H23" s="43" t="str"/>
+      <x:c r="I23" s="43" t="str"/>
+      <x:c r="J23" s="43" t="str"/>
+      <x:c r="K23" s="43" t="str"/>
+      <x:c r="L23" s="43" t="str"/>
+      <x:c r="M23" s="43" t="str"/>
+      <x:c r="N23" s="43" t="str"/>
+      <x:c r="O23" s="43" t="str"/>
+      <x:c r="P23" s="43" t="str"/>
+      <x:c r="Q23" s="43" t="str"/>
+      <x:c r="R23" s="43" t="str"/>
+      <x:c r="S23" s="43" t="str"/>
+      <x:c r="T23" s="43" t="str"/>
+      <x:c r="U23" s="43" t="str"/>
+      <x:c r="V23" s="43" t="str"/>
+      <x:c r="W23" s="43" t="str"/>
+      <x:c r="X23" s="43" t="str"/>
+      <x:c r="Y23" s="43" t="str"/>
+      <x:c r="Z23" s="43" t="str"/>
+      <x:c r="AA23" s="43" t="str"/>
+      <x:c r="AB23" s="43" t="str"/>
+      <x:c r="AC23" s="43" t="str"/>
+      <x:c r="AD23" s="43" t="str"/>
+      <x:c r="AE23" s="43" t="str"/>
+      <x:c r="AF23" s="43" t="str"/>
+      <x:c r="AG23" s="43" t="str"/>
+      <x:c r="AH23" s="43" t="str"/>
+      <x:c r="AI23" s="43" t="str"/>
+      <x:c r="AJ23" s="43" t="str"/>
+      <x:c r="AK23" s="43" t="str"/>
+      <x:c r="AL23" s="43" t="str"/>
+      <x:c r="AM23" s="43" t="str"/>
       <x:c r="AN23" s="32" t="str"/>
-      <x:c r="AO23" s="32" t="str"/>
-      <x:c r="AP23" s="32" t="str"/>
+      <x:c r="AO23" s="43" t="str"/>
+      <x:c r="AP23" s="43" t="str"/>
       <x:c r="AQ23" s="32" t="str"/>
-      <x:c r="AR23" s="32" t="str"/>
-      <x:c r="AS23" s="32" t="str"/>
+      <x:c r="AR23" s="43" t="str"/>
+      <x:c r="AS23" s="43" t="str"/>
       <x:c r="AT23" s="32" t="str"/>
       <x:c r="AU23" s="32" t="str"/>
       <x:c r="AV23" s="32" t="str"/>
-      <x:c r="AW23" s="33" t="str"/>
+      <x:c r="AW23" s="44" t="str"/>
       <x:c r="AX23" s="33" t="str"/>
       <x:c r="AY23" s="33" t="str"/>
       <x:c r="AZ23" s="33" t="str"/>
-      <x:c r="BA23" s="33" t="str">
+      <x:c r="BA23" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB23" s="33" t="str">
+      <x:c r="BB23" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC23" s="33" t="str">
+      <x:c r="BC23" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD23" s="33" t="str"/>
@@ -2321,58 +2332,58 @@
       <x:c r="E24" s="32" t="str"/>
       <x:c r="F24" s="32" t="str"/>
       <x:c r="G24" s="32" t="str"/>
-      <x:c r="H24" s="32" t="str"/>
-      <x:c r="I24" s="32" t="str"/>
-      <x:c r="J24" s="32" t="str"/>
-      <x:c r="K24" s="32" t="str"/>
-      <x:c r="L24" s="32" t="str"/>
-      <x:c r="M24" s="32" t="str"/>
-      <x:c r="N24" s="32" t="str"/>
-      <x:c r="O24" s="32" t="str"/>
-      <x:c r="P24" s="32" t="str"/>
-      <x:c r="Q24" s="32" t="str"/>
-      <x:c r="R24" s="32" t="str"/>
-      <x:c r="S24" s="32" t="str"/>
-      <x:c r="T24" s="32" t="str"/>
-      <x:c r="U24" s="32" t="str"/>
-      <x:c r="V24" s="32" t="str"/>
-      <x:c r="W24" s="32" t="str"/>
-      <x:c r="X24" s="32" t="str"/>
-      <x:c r="Y24" s="32" t="str"/>
-      <x:c r="Z24" s="32" t="str"/>
-      <x:c r="AA24" s="32" t="str"/>
-      <x:c r="AB24" s="32" t="str"/>
-      <x:c r="AC24" s="32" t="str"/>
-      <x:c r="AD24" s="32" t="str"/>
-      <x:c r="AE24" s="32" t="str"/>
-      <x:c r="AF24" s="32" t="str"/>
-      <x:c r="AG24" s="32" t="str"/>
-      <x:c r="AH24" s="32" t="str"/>
-      <x:c r="AI24" s="32" t="str"/>
-      <x:c r="AJ24" s="32" t="str"/>
-      <x:c r="AK24" s="32" t="str"/>
-      <x:c r="AL24" s="32" t="str"/>
-      <x:c r="AM24" s="32" t="str"/>
+      <x:c r="H24" s="43" t="str"/>
+      <x:c r="I24" s="43" t="str"/>
+      <x:c r="J24" s="43" t="str"/>
+      <x:c r="K24" s="43" t="str"/>
+      <x:c r="L24" s="43" t="str"/>
+      <x:c r="M24" s="43" t="str"/>
+      <x:c r="N24" s="43" t="str"/>
+      <x:c r="O24" s="43" t="str"/>
+      <x:c r="P24" s="43" t="str"/>
+      <x:c r="Q24" s="43" t="str"/>
+      <x:c r="R24" s="43" t="str"/>
+      <x:c r="S24" s="43" t="str"/>
+      <x:c r="T24" s="43" t="str"/>
+      <x:c r="U24" s="43" t="str"/>
+      <x:c r="V24" s="43" t="str"/>
+      <x:c r="W24" s="43" t="str"/>
+      <x:c r="X24" s="43" t="str"/>
+      <x:c r="Y24" s="43" t="str"/>
+      <x:c r="Z24" s="43" t="str"/>
+      <x:c r="AA24" s="43" t="str"/>
+      <x:c r="AB24" s="43" t="str"/>
+      <x:c r="AC24" s="43" t="str"/>
+      <x:c r="AD24" s="43" t="str"/>
+      <x:c r="AE24" s="43" t="str"/>
+      <x:c r="AF24" s="43" t="str"/>
+      <x:c r="AG24" s="43" t="str"/>
+      <x:c r="AH24" s="43" t="str"/>
+      <x:c r="AI24" s="43" t="str"/>
+      <x:c r="AJ24" s="43" t="str"/>
+      <x:c r="AK24" s="43" t="str"/>
+      <x:c r="AL24" s="43" t="str"/>
+      <x:c r="AM24" s="43" t="str"/>
       <x:c r="AN24" s="32" t="str"/>
-      <x:c r="AO24" s="32" t="str"/>
-      <x:c r="AP24" s="32" t="str"/>
+      <x:c r="AO24" s="43" t="str"/>
+      <x:c r="AP24" s="43" t="str"/>
       <x:c r="AQ24" s="32" t="str"/>
-      <x:c r="AR24" s="32" t="str"/>
-      <x:c r="AS24" s="32" t="str"/>
+      <x:c r="AR24" s="43" t="str"/>
+      <x:c r="AS24" s="43" t="str"/>
       <x:c r="AT24" s="32" t="str"/>
       <x:c r="AU24" s="32" t="str"/>
       <x:c r="AV24" s="32" t="str"/>
-      <x:c r="AW24" s="33" t="str"/>
+      <x:c r="AW24" s="44" t="str"/>
       <x:c r="AX24" s="33" t="str"/>
       <x:c r="AY24" s="33" t="str"/>
       <x:c r="AZ24" s="33" t="str"/>
-      <x:c r="BA24" s="33" t="str">
+      <x:c r="BA24" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB24" s="33" t="str">
+      <x:c r="BB24" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC24" s="33" t="str">
+      <x:c r="BC24" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD24" s="33" t="str"/>
@@ -2387,58 +2398,58 @@
       <x:c r="E25" s="32" t="str"/>
       <x:c r="F25" s="32" t="str"/>
       <x:c r="G25" s="32" t="str"/>
-      <x:c r="H25" s="32" t="str"/>
-      <x:c r="I25" s="32" t="str"/>
-      <x:c r="J25" s="32" t="str"/>
-      <x:c r="K25" s="32" t="str"/>
-      <x:c r="L25" s="32" t="str"/>
-      <x:c r="M25" s="32" t="str"/>
-      <x:c r="N25" s="32" t="str"/>
-      <x:c r="O25" s="32" t="str"/>
-      <x:c r="P25" s="32" t="str"/>
-      <x:c r="Q25" s="32" t="str"/>
-      <x:c r="R25" s="32" t="str"/>
-      <x:c r="S25" s="32" t="str"/>
-      <x:c r="T25" s="32" t="str"/>
-      <x:c r="U25" s="32" t="str"/>
-      <x:c r="V25" s="32" t="str"/>
-      <x:c r="W25" s="32" t="str"/>
-      <x:c r="X25" s="32" t="str"/>
-      <x:c r="Y25" s="32" t="str"/>
-      <x:c r="Z25" s="32" t="str"/>
-      <x:c r="AA25" s="32" t="str"/>
-      <x:c r="AB25" s="32" t="str"/>
-      <x:c r="AC25" s="32" t="str"/>
-      <x:c r="AD25" s="32" t="str"/>
-      <x:c r="AE25" s="32" t="str"/>
-      <x:c r="AF25" s="32" t="str"/>
-      <x:c r="AG25" s="32" t="str"/>
-      <x:c r="AH25" s="32" t="str"/>
-      <x:c r="AI25" s="32" t="str"/>
-      <x:c r="AJ25" s="32" t="str"/>
-      <x:c r="AK25" s="32" t="str"/>
-      <x:c r="AL25" s="32" t="str"/>
-      <x:c r="AM25" s="32" t="str"/>
+      <x:c r="H25" s="43" t="str"/>
+      <x:c r="I25" s="43" t="str"/>
+      <x:c r="J25" s="43" t="str"/>
+      <x:c r="K25" s="43" t="str"/>
+      <x:c r="L25" s="43" t="str"/>
+      <x:c r="M25" s="43" t="str"/>
+      <x:c r="N25" s="43" t="str"/>
+      <x:c r="O25" s="43" t="str"/>
+      <x:c r="P25" s="43" t="str"/>
+      <x:c r="Q25" s="43" t="str"/>
+      <x:c r="R25" s="43" t="str"/>
+      <x:c r="S25" s="43" t="str"/>
+      <x:c r="T25" s="43" t="str"/>
+      <x:c r="U25" s="43" t="str"/>
+      <x:c r="V25" s="43" t="str"/>
+      <x:c r="W25" s="43" t="str"/>
+      <x:c r="X25" s="43" t="str"/>
+      <x:c r="Y25" s="43" t="str"/>
+      <x:c r="Z25" s="43" t="str"/>
+      <x:c r="AA25" s="43" t="str"/>
+      <x:c r="AB25" s="43" t="str"/>
+      <x:c r="AC25" s="43" t="str"/>
+      <x:c r="AD25" s="43" t="str"/>
+      <x:c r="AE25" s="43" t="str"/>
+      <x:c r="AF25" s="43" t="str"/>
+      <x:c r="AG25" s="43" t="str"/>
+      <x:c r="AH25" s="43" t="str"/>
+      <x:c r="AI25" s="43" t="str"/>
+      <x:c r="AJ25" s="43" t="str"/>
+      <x:c r="AK25" s="43" t="str"/>
+      <x:c r="AL25" s="43" t="str"/>
+      <x:c r="AM25" s="43" t="str"/>
       <x:c r="AN25" s="32" t="str"/>
-      <x:c r="AO25" s="32" t="str"/>
-      <x:c r="AP25" s="32" t="str"/>
+      <x:c r="AO25" s="43" t="str"/>
+      <x:c r="AP25" s="43" t="str"/>
       <x:c r="AQ25" s="32" t="str"/>
-      <x:c r="AR25" s="32" t="str"/>
-      <x:c r="AS25" s="32" t="str"/>
+      <x:c r="AR25" s="43" t="str"/>
+      <x:c r="AS25" s="43" t="str"/>
       <x:c r="AT25" s="32" t="str"/>
       <x:c r="AU25" s="32" t="str"/>
       <x:c r="AV25" s="32" t="str"/>
-      <x:c r="AW25" s="33" t="str"/>
+      <x:c r="AW25" s="44" t="str"/>
       <x:c r="AX25" s="33" t="str"/>
       <x:c r="AY25" s="33" t="str"/>
       <x:c r="AZ25" s="33" t="str"/>
-      <x:c r="BA25" s="33" t="str">
+      <x:c r="BA25" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB25" s="33" t="str">
+      <x:c r="BB25" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC25" s="33" t="str">
+      <x:c r="BC25" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD25" s="33" t="str"/>
@@ -2453,58 +2464,58 @@
       <x:c r="E26" s="32" t="str"/>
       <x:c r="F26" s="32" t="str"/>
       <x:c r="G26" s="32" t="str"/>
-      <x:c r="H26" s="32" t="str"/>
-      <x:c r="I26" s="32" t="str"/>
-      <x:c r="J26" s="32" t="str"/>
-      <x:c r="K26" s="32" t="str"/>
-      <x:c r="L26" s="32" t="str"/>
-      <x:c r="M26" s="32" t="str"/>
-      <x:c r="N26" s="32" t="str"/>
-      <x:c r="O26" s="32" t="str"/>
-      <x:c r="P26" s="32" t="str"/>
-      <x:c r="Q26" s="32" t="str"/>
-      <x:c r="R26" s="32" t="str"/>
-      <x:c r="S26" s="32" t="str"/>
-      <x:c r="T26" s="32" t="str"/>
-      <x:c r="U26" s="32" t="str"/>
-      <x:c r="V26" s="32" t="str"/>
-      <x:c r="W26" s="32" t="str"/>
-      <x:c r="X26" s="32" t="str"/>
-      <x:c r="Y26" s="32" t="str"/>
-      <x:c r="Z26" s="32" t="str"/>
-      <x:c r="AA26" s="32" t="str"/>
-      <x:c r="AB26" s="32" t="str"/>
-      <x:c r="AC26" s="32" t="str"/>
-      <x:c r="AD26" s="32" t="str"/>
-      <x:c r="AE26" s="32" t="str"/>
-      <x:c r="AF26" s="32" t="str"/>
-      <x:c r="AG26" s="32" t="str"/>
-      <x:c r="AH26" s="32" t="str"/>
-      <x:c r="AI26" s="32" t="str"/>
-      <x:c r="AJ26" s="32" t="str"/>
-      <x:c r="AK26" s="32" t="str"/>
-      <x:c r="AL26" s="32" t="str"/>
-      <x:c r="AM26" s="32" t="str"/>
+      <x:c r="H26" s="43" t="str"/>
+      <x:c r="I26" s="43" t="str"/>
+      <x:c r="J26" s="43" t="str"/>
+      <x:c r="K26" s="43" t="str"/>
+      <x:c r="L26" s="43" t="str"/>
+      <x:c r="M26" s="43" t="str"/>
+      <x:c r="N26" s="43" t="str"/>
+      <x:c r="O26" s="43" t="str"/>
+      <x:c r="P26" s="43" t="str"/>
+      <x:c r="Q26" s="43" t="str"/>
+      <x:c r="R26" s="43" t="str"/>
+      <x:c r="S26" s="43" t="str"/>
+      <x:c r="T26" s="43" t="str"/>
+      <x:c r="U26" s="43" t="str"/>
+      <x:c r="V26" s="43" t="str"/>
+      <x:c r="W26" s="43" t="str"/>
+      <x:c r="X26" s="43" t="str"/>
+      <x:c r="Y26" s="43" t="str"/>
+      <x:c r="Z26" s="43" t="str"/>
+      <x:c r="AA26" s="43" t="str"/>
+      <x:c r="AB26" s="43" t="str"/>
+      <x:c r="AC26" s="43" t="str"/>
+      <x:c r="AD26" s="43" t="str"/>
+      <x:c r="AE26" s="43" t="str"/>
+      <x:c r="AF26" s="43" t="str"/>
+      <x:c r="AG26" s="43" t="str"/>
+      <x:c r="AH26" s="43" t="str"/>
+      <x:c r="AI26" s="43" t="str"/>
+      <x:c r="AJ26" s="43" t="str"/>
+      <x:c r="AK26" s="43" t="str"/>
+      <x:c r="AL26" s="43" t="str"/>
+      <x:c r="AM26" s="43" t="str"/>
       <x:c r="AN26" s="32" t="str"/>
-      <x:c r="AO26" s="32" t="str"/>
-      <x:c r="AP26" s="32" t="str"/>
+      <x:c r="AO26" s="43" t="str"/>
+      <x:c r="AP26" s="43" t="str"/>
       <x:c r="AQ26" s="32" t="str"/>
-      <x:c r="AR26" s="32" t="str"/>
-      <x:c r="AS26" s="32" t="str"/>
+      <x:c r="AR26" s="43" t="str"/>
+      <x:c r="AS26" s="43" t="str"/>
       <x:c r="AT26" s="32" t="str"/>
       <x:c r="AU26" s="32" t="str"/>
       <x:c r="AV26" s="32" t="str"/>
-      <x:c r="AW26" s="33" t="str"/>
+      <x:c r="AW26" s="44" t="str"/>
       <x:c r="AX26" s="33" t="str"/>
       <x:c r="AY26" s="33" t="str"/>
       <x:c r="AZ26" s="33" t="str"/>
-      <x:c r="BA26" s="33" t="str">
+      <x:c r="BA26" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB26" s="33" t="str">
+      <x:c r="BB26" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC26" s="33" t="str">
+      <x:c r="BC26" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD26" s="33" t="str"/>
@@ -2519,58 +2530,58 @@
       <x:c r="E27" s="32" t="str"/>
       <x:c r="F27" s="32" t="str"/>
       <x:c r="G27" s="32" t="str"/>
-      <x:c r="H27" s="32" t="str"/>
-      <x:c r="I27" s="32" t="str"/>
-      <x:c r="J27" s="32" t="str"/>
-      <x:c r="K27" s="32" t="str"/>
-      <x:c r="L27" s="32" t="str"/>
-      <x:c r="M27" s="32" t="str"/>
-      <x:c r="N27" s="32" t="str"/>
-      <x:c r="O27" s="32" t="str"/>
-      <x:c r="P27" s="32" t="str"/>
-      <x:c r="Q27" s="32" t="str"/>
-      <x:c r="R27" s="32" t="str"/>
-      <x:c r="S27" s="32" t="str"/>
-      <x:c r="T27" s="32" t="str"/>
-      <x:c r="U27" s="32" t="str"/>
-      <x:c r="V27" s="32" t="str"/>
-      <x:c r="W27" s="32" t="str"/>
-      <x:c r="X27" s="32" t="str"/>
-      <x:c r="Y27" s="32" t="str"/>
-      <x:c r="Z27" s="32" t="str"/>
-      <x:c r="AA27" s="32" t="str"/>
-      <x:c r="AB27" s="32" t="str"/>
-      <x:c r="AC27" s="32" t="str"/>
-      <x:c r="AD27" s="32" t="str"/>
-      <x:c r="AE27" s="32" t="str"/>
-      <x:c r="AF27" s="32" t="str"/>
-      <x:c r="AG27" s="32" t="str"/>
-      <x:c r="AH27" s="32" t="str"/>
-      <x:c r="AI27" s="32" t="str"/>
-      <x:c r="AJ27" s="32" t="str"/>
-      <x:c r="AK27" s="32" t="str"/>
-      <x:c r="AL27" s="32" t="str"/>
-      <x:c r="AM27" s="32" t="str"/>
+      <x:c r="H27" s="43" t="str"/>
+      <x:c r="I27" s="43" t="str"/>
+      <x:c r="J27" s="43" t="str"/>
+      <x:c r="K27" s="43" t="str"/>
+      <x:c r="L27" s="43" t="str"/>
+      <x:c r="M27" s="43" t="str"/>
+      <x:c r="N27" s="43" t="str"/>
+      <x:c r="O27" s="43" t="str"/>
+      <x:c r="P27" s="43" t="str"/>
+      <x:c r="Q27" s="43" t="str"/>
+      <x:c r="R27" s="43" t="str"/>
+      <x:c r="S27" s="43" t="str"/>
+      <x:c r="T27" s="43" t="str"/>
+      <x:c r="U27" s="43" t="str"/>
+      <x:c r="V27" s="43" t="str"/>
+      <x:c r="W27" s="43" t="str"/>
+      <x:c r="X27" s="43" t="str"/>
+      <x:c r="Y27" s="43" t="str"/>
+      <x:c r="Z27" s="43" t="str"/>
+      <x:c r="AA27" s="43" t="str"/>
+      <x:c r="AB27" s="43" t="str"/>
+      <x:c r="AC27" s="43" t="str"/>
+      <x:c r="AD27" s="43" t="str"/>
+      <x:c r="AE27" s="43" t="str"/>
+      <x:c r="AF27" s="43" t="str"/>
+      <x:c r="AG27" s="43" t="str"/>
+      <x:c r="AH27" s="43" t="str"/>
+      <x:c r="AI27" s="43" t="str"/>
+      <x:c r="AJ27" s="43" t="str"/>
+      <x:c r="AK27" s="43" t="str"/>
+      <x:c r="AL27" s="43" t="str"/>
+      <x:c r="AM27" s="43" t="str"/>
       <x:c r="AN27" s="32" t="str"/>
-      <x:c r="AO27" s="32" t="str"/>
-      <x:c r="AP27" s="32" t="str"/>
+      <x:c r="AO27" s="43" t="str"/>
+      <x:c r="AP27" s="43" t="str"/>
       <x:c r="AQ27" s="32" t="str"/>
-      <x:c r="AR27" s="32" t="str"/>
-      <x:c r="AS27" s="32" t="str"/>
+      <x:c r="AR27" s="43" t="str"/>
+      <x:c r="AS27" s="43" t="str"/>
       <x:c r="AT27" s="32" t="str"/>
       <x:c r="AU27" s="32" t="str"/>
       <x:c r="AV27" s="32" t="str"/>
-      <x:c r="AW27" s="33" t="str"/>
+      <x:c r="AW27" s="44" t="str"/>
       <x:c r="AX27" s="33" t="str"/>
       <x:c r="AY27" s="33" t="str"/>
       <x:c r="AZ27" s="33" t="str"/>
-      <x:c r="BA27" s="33" t="str">
+      <x:c r="BA27" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB27" s="33" t="str">
+      <x:c r="BB27" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC27" s="33" t="str">
+      <x:c r="BC27" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD27" s="33" t="str"/>
@@ -2585,58 +2596,58 @@
       <x:c r="E28" s="32" t="str"/>
       <x:c r="F28" s="32" t="str"/>
       <x:c r="G28" s="32" t="str"/>
-      <x:c r="H28" s="32" t="str"/>
-      <x:c r="I28" s="32" t="str"/>
-      <x:c r="J28" s="32" t="str"/>
-      <x:c r="K28" s="32" t="str"/>
-      <x:c r="L28" s="32" t="str"/>
-      <x:c r="M28" s="32" t="str"/>
-      <x:c r="N28" s="32" t="str"/>
-      <x:c r="O28" s="32" t="str"/>
-      <x:c r="P28" s="32" t="str"/>
-      <x:c r="Q28" s="32" t="str"/>
-      <x:c r="R28" s="32" t="str"/>
-      <x:c r="S28" s="32" t="str"/>
-      <x:c r="T28" s="32" t="str"/>
-      <x:c r="U28" s="32" t="str"/>
-      <x:c r="V28" s="32" t="str"/>
-      <x:c r="W28" s="32" t="str"/>
-      <x:c r="X28" s="32" t="str"/>
-      <x:c r="Y28" s="32" t="str"/>
-      <x:c r="Z28" s="32" t="str"/>
-      <x:c r="AA28" s="32" t="str"/>
-      <x:c r="AB28" s="32" t="str"/>
-      <x:c r="AC28" s="32" t="str"/>
-      <x:c r="AD28" s="32" t="str"/>
-      <x:c r="AE28" s="32" t="str"/>
-      <x:c r="AF28" s="32" t="str"/>
-      <x:c r="AG28" s="32" t="str"/>
-      <x:c r="AH28" s="32" t="str"/>
-      <x:c r="AI28" s="32" t="str"/>
-      <x:c r="AJ28" s="32" t="str"/>
-      <x:c r="AK28" s="32" t="str"/>
-      <x:c r="AL28" s="32" t="str"/>
-      <x:c r="AM28" s="32" t="str"/>
+      <x:c r="H28" s="43" t="str"/>
+      <x:c r="I28" s="43" t="str"/>
+      <x:c r="J28" s="43" t="str"/>
+      <x:c r="K28" s="43" t="str"/>
+      <x:c r="L28" s="43" t="str"/>
+      <x:c r="M28" s="43" t="str"/>
+      <x:c r="N28" s="43" t="str"/>
+      <x:c r="O28" s="43" t="str"/>
+      <x:c r="P28" s="43" t="str"/>
+      <x:c r="Q28" s="43" t="str"/>
+      <x:c r="R28" s="43" t="str"/>
+      <x:c r="S28" s="43" t="str"/>
+      <x:c r="T28" s="43" t="str"/>
+      <x:c r="U28" s="43" t="str"/>
+      <x:c r="V28" s="43" t="str"/>
+      <x:c r="W28" s="43" t="str"/>
+      <x:c r="X28" s="43" t="str"/>
+      <x:c r="Y28" s="43" t="str"/>
+      <x:c r="Z28" s="43" t="str"/>
+      <x:c r="AA28" s="43" t="str"/>
+      <x:c r="AB28" s="43" t="str"/>
+      <x:c r="AC28" s="43" t="str"/>
+      <x:c r="AD28" s="43" t="str"/>
+      <x:c r="AE28" s="43" t="str"/>
+      <x:c r="AF28" s="43" t="str"/>
+      <x:c r="AG28" s="43" t="str"/>
+      <x:c r="AH28" s="43" t="str"/>
+      <x:c r="AI28" s="43" t="str"/>
+      <x:c r="AJ28" s="43" t="str"/>
+      <x:c r="AK28" s="43" t="str"/>
+      <x:c r="AL28" s="43" t="str"/>
+      <x:c r="AM28" s="43" t="str"/>
       <x:c r="AN28" s="32" t="str"/>
-      <x:c r="AO28" s="32" t="str"/>
-      <x:c r="AP28" s="32" t="str"/>
+      <x:c r="AO28" s="43" t="str"/>
+      <x:c r="AP28" s="43" t="str"/>
       <x:c r="AQ28" s="32" t="str"/>
-      <x:c r="AR28" s="32" t="str"/>
-      <x:c r="AS28" s="32" t="str"/>
+      <x:c r="AR28" s="43" t="str"/>
+      <x:c r="AS28" s="43" t="str"/>
       <x:c r="AT28" s="32" t="str"/>
       <x:c r="AU28" s="32" t="str"/>
       <x:c r="AV28" s="32" t="str"/>
-      <x:c r="AW28" s="33" t="str"/>
+      <x:c r="AW28" s="44" t="str"/>
       <x:c r="AX28" s="33" t="str"/>
       <x:c r="AY28" s="33" t="str"/>
       <x:c r="AZ28" s="33" t="str"/>
-      <x:c r="BA28" s="33" t="str">
+      <x:c r="BA28" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB28" s="33" t="str">
+      <x:c r="BB28" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC28" s="33" t="str">
+      <x:c r="BC28" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD28" s="33" t="str"/>
@@ -2651,58 +2662,58 @@
       <x:c r="E29" s="32" t="str"/>
       <x:c r="F29" s="32" t="str"/>
       <x:c r="G29" s="32" t="str"/>
-      <x:c r="H29" s="32" t="str"/>
-      <x:c r="I29" s="32" t="str"/>
-      <x:c r="J29" s="32" t="str"/>
-      <x:c r="K29" s="32" t="str"/>
-      <x:c r="L29" s="32" t="str"/>
-      <x:c r="M29" s="32" t="str"/>
-      <x:c r="N29" s="32" t="str"/>
-      <x:c r="O29" s="32" t="str"/>
-      <x:c r="P29" s="32" t="str"/>
-      <x:c r="Q29" s="32" t="str"/>
-      <x:c r="R29" s="32" t="str"/>
-      <x:c r="S29" s="32" t="str"/>
-      <x:c r="T29" s="32" t="str"/>
-      <x:c r="U29" s="32" t="str"/>
-      <x:c r="V29" s="32" t="str"/>
-      <x:c r="W29" s="32" t="str"/>
-      <x:c r="X29" s="32" t="str"/>
-      <x:c r="Y29" s="32" t="str"/>
-      <x:c r="Z29" s="32" t="str"/>
-      <x:c r="AA29" s="32" t="str"/>
-      <x:c r="AB29" s="32" t="str"/>
-      <x:c r="AC29" s="32" t="str"/>
-      <x:c r="AD29" s="32" t="str"/>
-      <x:c r="AE29" s="32" t="str"/>
-      <x:c r="AF29" s="32" t="str"/>
-      <x:c r="AG29" s="32" t="str"/>
-      <x:c r="AH29" s="32" t="str"/>
-      <x:c r="AI29" s="32" t="str"/>
-      <x:c r="AJ29" s="32" t="str"/>
-      <x:c r="AK29" s="32" t="str"/>
-      <x:c r="AL29" s="32" t="str"/>
-      <x:c r="AM29" s="32" t="str"/>
+      <x:c r="H29" s="43" t="str"/>
+      <x:c r="I29" s="43" t="str"/>
+      <x:c r="J29" s="43" t="str"/>
+      <x:c r="K29" s="43" t="str"/>
+      <x:c r="L29" s="43" t="str"/>
+      <x:c r="M29" s="43" t="str"/>
+      <x:c r="N29" s="43" t="str"/>
+      <x:c r="O29" s="43" t="str"/>
+      <x:c r="P29" s="43" t="str"/>
+      <x:c r="Q29" s="43" t="str"/>
+      <x:c r="R29" s="43" t="str"/>
+      <x:c r="S29" s="43" t="str"/>
+      <x:c r="T29" s="43" t="str"/>
+      <x:c r="U29" s="43" t="str"/>
+      <x:c r="V29" s="43" t="str"/>
+      <x:c r="W29" s="43" t="str"/>
+      <x:c r="X29" s="43" t="str"/>
+      <x:c r="Y29" s="43" t="str"/>
+      <x:c r="Z29" s="43" t="str"/>
+      <x:c r="AA29" s="43" t="str"/>
+      <x:c r="AB29" s="43" t="str"/>
+      <x:c r="AC29" s="43" t="str"/>
+      <x:c r="AD29" s="43" t="str"/>
+      <x:c r="AE29" s="43" t="str"/>
+      <x:c r="AF29" s="43" t="str"/>
+      <x:c r="AG29" s="43" t="str"/>
+      <x:c r="AH29" s="43" t="str"/>
+      <x:c r="AI29" s="43" t="str"/>
+      <x:c r="AJ29" s="43" t="str"/>
+      <x:c r="AK29" s="43" t="str"/>
+      <x:c r="AL29" s="43" t="str"/>
+      <x:c r="AM29" s="43" t="str"/>
       <x:c r="AN29" s="32" t="str"/>
-      <x:c r="AO29" s="32" t="str"/>
-      <x:c r="AP29" s="32" t="str"/>
+      <x:c r="AO29" s="43" t="str"/>
+      <x:c r="AP29" s="43" t="str"/>
       <x:c r="AQ29" s="32" t="str"/>
-      <x:c r="AR29" s="32" t="str"/>
-      <x:c r="AS29" s="32" t="str"/>
+      <x:c r="AR29" s="43" t="str"/>
+      <x:c r="AS29" s="43" t="str"/>
       <x:c r="AT29" s="32" t="str"/>
       <x:c r="AU29" s="32" t="str"/>
       <x:c r="AV29" s="32" t="str"/>
-      <x:c r="AW29" s="33" t="str"/>
+      <x:c r="AW29" s="44" t="str"/>
       <x:c r="AX29" s="33" t="str"/>
       <x:c r="AY29" s="33" t="str"/>
       <x:c r="AZ29" s="33" t="str"/>
-      <x:c r="BA29" s="33" t="str">
+      <x:c r="BA29" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB29" s="33" t="str">
+      <x:c r="BB29" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC29" s="33" t="str">
+      <x:c r="BC29" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD29" s="33" t="str"/>
@@ -2717,58 +2728,58 @@
       <x:c r="E30" s="32" t="str"/>
       <x:c r="F30" s="32" t="str"/>
       <x:c r="G30" s="32" t="str"/>
-      <x:c r="H30" s="32" t="str"/>
-      <x:c r="I30" s="32" t="str"/>
-      <x:c r="J30" s="32" t="str"/>
-      <x:c r="K30" s="32" t="str"/>
-      <x:c r="L30" s="32" t="str"/>
-      <x:c r="M30" s="32" t="str"/>
-      <x:c r="N30" s="32" t="str"/>
-      <x:c r="O30" s="32" t="str"/>
-      <x:c r="P30" s="32" t="str"/>
-      <x:c r="Q30" s="32" t="str"/>
-      <x:c r="R30" s="32" t="str"/>
-      <x:c r="S30" s="32" t="str"/>
-      <x:c r="T30" s="32" t="str"/>
-      <x:c r="U30" s="32" t="str"/>
-      <x:c r="V30" s="32" t="str"/>
-      <x:c r="W30" s="32" t="str"/>
-      <x:c r="X30" s="32" t="str"/>
-      <x:c r="Y30" s="32" t="str"/>
-      <x:c r="Z30" s="32" t="str"/>
-      <x:c r="AA30" s="32" t="str"/>
-      <x:c r="AB30" s="32" t="str"/>
-      <x:c r="AC30" s="32" t="str"/>
-      <x:c r="AD30" s="32" t="str"/>
-      <x:c r="AE30" s="32" t="str"/>
-      <x:c r="AF30" s="32" t="str"/>
-      <x:c r="AG30" s="32" t="str"/>
-      <x:c r="AH30" s="32" t="str"/>
-      <x:c r="AI30" s="32" t="str"/>
-      <x:c r="AJ30" s="32" t="str"/>
-      <x:c r="AK30" s="32" t="str"/>
-      <x:c r="AL30" s="32" t="str"/>
-      <x:c r="AM30" s="32" t="str"/>
+      <x:c r="H30" s="43" t="str"/>
+      <x:c r="I30" s="43" t="str"/>
+      <x:c r="J30" s="43" t="str"/>
+      <x:c r="K30" s="43" t="str"/>
+      <x:c r="L30" s="43" t="str"/>
+      <x:c r="M30" s="43" t="str"/>
+      <x:c r="N30" s="43" t="str"/>
+      <x:c r="O30" s="43" t="str"/>
+      <x:c r="P30" s="43" t="str"/>
+      <x:c r="Q30" s="43" t="str"/>
+      <x:c r="R30" s="43" t="str"/>
+      <x:c r="S30" s="43" t="str"/>
+      <x:c r="T30" s="43" t="str"/>
+      <x:c r="U30" s="43" t="str"/>
+      <x:c r="V30" s="43" t="str"/>
+      <x:c r="W30" s="43" t="str"/>
+      <x:c r="X30" s="43" t="str"/>
+      <x:c r="Y30" s="43" t="str"/>
+      <x:c r="Z30" s="43" t="str"/>
+      <x:c r="AA30" s="43" t="str"/>
+      <x:c r="AB30" s="43" t="str"/>
+      <x:c r="AC30" s="43" t="str"/>
+      <x:c r="AD30" s="43" t="str"/>
+      <x:c r="AE30" s="43" t="str"/>
+      <x:c r="AF30" s="43" t="str"/>
+      <x:c r="AG30" s="43" t="str"/>
+      <x:c r="AH30" s="43" t="str"/>
+      <x:c r="AI30" s="43" t="str"/>
+      <x:c r="AJ30" s="43" t="str"/>
+      <x:c r="AK30" s="43" t="str"/>
+      <x:c r="AL30" s="43" t="str"/>
+      <x:c r="AM30" s="43" t="str"/>
       <x:c r="AN30" s="32" t="str"/>
-      <x:c r="AO30" s="32" t="str"/>
-      <x:c r="AP30" s="32" t="str"/>
+      <x:c r="AO30" s="43" t="str"/>
+      <x:c r="AP30" s="43" t="str"/>
       <x:c r="AQ30" s="32" t="str"/>
-      <x:c r="AR30" s="32" t="str"/>
-      <x:c r="AS30" s="32" t="str"/>
+      <x:c r="AR30" s="43" t="str"/>
+      <x:c r="AS30" s="43" t="str"/>
       <x:c r="AT30" s="32" t="str"/>
       <x:c r="AU30" s="32" t="str"/>
       <x:c r="AV30" s="32" t="str"/>
-      <x:c r="AW30" s="33" t="str"/>
+      <x:c r="AW30" s="44" t="str"/>
       <x:c r="AX30" s="33" t="str"/>
       <x:c r="AY30" s="33" t="str"/>
       <x:c r="AZ30" s="33" t="str"/>
-      <x:c r="BA30" s="33" t="str">
+      <x:c r="BA30" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB30" s="33" t="str">
+      <x:c r="BB30" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC30" s="33" t="str">
+      <x:c r="BC30" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD30" s="33" t="str"/>
@@ -2783,58 +2794,58 @@
       <x:c r="E31" s="32" t="str"/>
       <x:c r="F31" s="32" t="str"/>
       <x:c r="G31" s="32" t="str"/>
-      <x:c r="H31" s="32" t="str"/>
-      <x:c r="I31" s="32" t="str"/>
-      <x:c r="J31" s="32" t="str"/>
-      <x:c r="K31" s="32" t="str"/>
-      <x:c r="L31" s="32" t="str"/>
-      <x:c r="M31" s="32" t="str"/>
-      <x:c r="N31" s="32" t="str"/>
-      <x:c r="O31" s="32" t="str"/>
-      <x:c r="P31" s="32" t="str"/>
-      <x:c r="Q31" s="32" t="str"/>
-      <x:c r="R31" s="32" t="str"/>
-      <x:c r="S31" s="32" t="str"/>
-      <x:c r="T31" s="32" t="str"/>
-      <x:c r="U31" s="32" t="str"/>
-      <x:c r="V31" s="32" t="str"/>
-      <x:c r="W31" s="32" t="str"/>
-      <x:c r="X31" s="32" t="str"/>
-      <x:c r="Y31" s="32" t="str"/>
-      <x:c r="Z31" s="32" t="str"/>
-      <x:c r="AA31" s="32" t="str"/>
-      <x:c r="AB31" s="32" t="str"/>
-      <x:c r="AC31" s="32" t="str"/>
-      <x:c r="AD31" s="32" t="str"/>
-      <x:c r="AE31" s="32" t="str"/>
-      <x:c r="AF31" s="32" t="str"/>
-      <x:c r="AG31" s="32" t="str"/>
-      <x:c r="AH31" s="32" t="str"/>
-      <x:c r="AI31" s="32" t="str"/>
-      <x:c r="AJ31" s="32" t="str"/>
-      <x:c r="AK31" s="32" t="str"/>
-      <x:c r="AL31" s="32" t="str"/>
-      <x:c r="AM31" s="32" t="str"/>
+      <x:c r="H31" s="43" t="str"/>
+      <x:c r="I31" s="43" t="str"/>
+      <x:c r="J31" s="43" t="str"/>
+      <x:c r="K31" s="43" t="str"/>
+      <x:c r="L31" s="43" t="str"/>
+      <x:c r="M31" s="43" t="str"/>
+      <x:c r="N31" s="43" t="str"/>
+      <x:c r="O31" s="43" t="str"/>
+      <x:c r="P31" s="43" t="str"/>
+      <x:c r="Q31" s="43" t="str"/>
+      <x:c r="R31" s="43" t="str"/>
+      <x:c r="S31" s="43" t="str"/>
+      <x:c r="T31" s="43" t="str"/>
+      <x:c r="U31" s="43" t="str"/>
+      <x:c r="V31" s="43" t="str"/>
+      <x:c r="W31" s="43" t="str"/>
+      <x:c r="X31" s="43" t="str"/>
+      <x:c r="Y31" s="43" t="str"/>
+      <x:c r="Z31" s="43" t="str"/>
+      <x:c r="AA31" s="43" t="str"/>
+      <x:c r="AB31" s="43" t="str"/>
+      <x:c r="AC31" s="43" t="str"/>
+      <x:c r="AD31" s="43" t="str"/>
+      <x:c r="AE31" s="43" t="str"/>
+      <x:c r="AF31" s="43" t="str"/>
+      <x:c r="AG31" s="43" t="str"/>
+      <x:c r="AH31" s="43" t="str"/>
+      <x:c r="AI31" s="43" t="str"/>
+      <x:c r="AJ31" s="43" t="str"/>
+      <x:c r="AK31" s="43" t="str"/>
+      <x:c r="AL31" s="43" t="str"/>
+      <x:c r="AM31" s="43" t="str"/>
       <x:c r="AN31" s="32" t="str"/>
-      <x:c r="AO31" s="32" t="str"/>
-      <x:c r="AP31" s="32" t="str"/>
+      <x:c r="AO31" s="43" t="str"/>
+      <x:c r="AP31" s="43" t="str"/>
       <x:c r="AQ31" s="32" t="str"/>
-      <x:c r="AR31" s="32" t="str"/>
-      <x:c r="AS31" s="32" t="str"/>
+      <x:c r="AR31" s="43" t="str"/>
+      <x:c r="AS31" s="43" t="str"/>
       <x:c r="AT31" s="32" t="str"/>
       <x:c r="AU31" s="32" t="str"/>
       <x:c r="AV31" s="32" t="str"/>
-      <x:c r="AW31" s="33" t="str"/>
+      <x:c r="AW31" s="44" t="str"/>
       <x:c r="AX31" s="33" t="str"/>
       <x:c r="AY31" s="33" t="str"/>
       <x:c r="AZ31" s="33" t="str"/>
-      <x:c r="BA31" s="33" t="str">
+      <x:c r="BA31" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB31" s="33" t="str">
+      <x:c r="BB31" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC31" s="33" t="str">
+      <x:c r="BC31" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD31" s="33" t="str"/>
@@ -2849,58 +2860,58 @@
       <x:c r="E32" s="32" t="str"/>
       <x:c r="F32" s="32" t="str"/>
       <x:c r="G32" s="32" t="str"/>
-      <x:c r="H32" s="32" t="str"/>
-      <x:c r="I32" s="32" t="str"/>
-      <x:c r="J32" s="32" t="str"/>
-      <x:c r="K32" s="32" t="str"/>
-      <x:c r="L32" s="32" t="str"/>
-      <x:c r="M32" s="32" t="str"/>
-      <x:c r="N32" s="32" t="str"/>
-      <x:c r="O32" s="32" t="str"/>
-      <x:c r="P32" s="32" t="str"/>
-      <x:c r="Q32" s="32" t="str"/>
-      <x:c r="R32" s="32" t="str"/>
-      <x:c r="S32" s="32" t="str"/>
-      <x:c r="T32" s="32" t="str"/>
-      <x:c r="U32" s="32" t="str"/>
-      <x:c r="V32" s="32" t="str"/>
-      <x:c r="W32" s="32" t="str"/>
-      <x:c r="X32" s="32" t="str"/>
-      <x:c r="Y32" s="32" t="str"/>
-      <x:c r="Z32" s="32" t="str"/>
-      <x:c r="AA32" s="32" t="str"/>
-      <x:c r="AB32" s="32" t="str"/>
-      <x:c r="AC32" s="32" t="str"/>
-      <x:c r="AD32" s="32" t="str"/>
-      <x:c r="AE32" s="32" t="str"/>
-      <x:c r="AF32" s="32" t="str"/>
-      <x:c r="AG32" s="32" t="str"/>
-      <x:c r="AH32" s="32" t="str"/>
-      <x:c r="AI32" s="32" t="str"/>
-      <x:c r="AJ32" s="32" t="str"/>
-      <x:c r="AK32" s="32" t="str"/>
-      <x:c r="AL32" s="32" t="str"/>
-      <x:c r="AM32" s="32" t="str"/>
+      <x:c r="H32" s="43" t="str"/>
+      <x:c r="I32" s="43" t="str"/>
+      <x:c r="J32" s="43" t="str"/>
+      <x:c r="K32" s="43" t="str"/>
+      <x:c r="L32" s="43" t="str"/>
+      <x:c r="M32" s="43" t="str"/>
+      <x:c r="N32" s="43" t="str"/>
+      <x:c r="O32" s="43" t="str"/>
+      <x:c r="P32" s="43" t="str"/>
+      <x:c r="Q32" s="43" t="str"/>
+      <x:c r="R32" s="43" t="str"/>
+      <x:c r="S32" s="43" t="str"/>
+      <x:c r="T32" s="43" t="str"/>
+      <x:c r="U32" s="43" t="str"/>
+      <x:c r="V32" s="43" t="str"/>
+      <x:c r="W32" s="43" t="str"/>
+      <x:c r="X32" s="43" t="str"/>
+      <x:c r="Y32" s="43" t="str"/>
+      <x:c r="Z32" s="43" t="str"/>
+      <x:c r="AA32" s="43" t="str"/>
+      <x:c r="AB32" s="43" t="str"/>
+      <x:c r="AC32" s="43" t="str"/>
+      <x:c r="AD32" s="43" t="str"/>
+      <x:c r="AE32" s="43" t="str"/>
+      <x:c r="AF32" s="43" t="str"/>
+      <x:c r="AG32" s="43" t="str"/>
+      <x:c r="AH32" s="43" t="str"/>
+      <x:c r="AI32" s="43" t="str"/>
+      <x:c r="AJ32" s="43" t="str"/>
+      <x:c r="AK32" s="43" t="str"/>
+      <x:c r="AL32" s="43" t="str"/>
+      <x:c r="AM32" s="43" t="str"/>
       <x:c r="AN32" s="32" t="str"/>
-      <x:c r="AO32" s="32" t="str"/>
-      <x:c r="AP32" s="32" t="str"/>
+      <x:c r="AO32" s="43" t="str"/>
+      <x:c r="AP32" s="43" t="str"/>
       <x:c r="AQ32" s="32" t="str"/>
-      <x:c r="AR32" s="32" t="str"/>
-      <x:c r="AS32" s="32" t="str"/>
+      <x:c r="AR32" s="43" t="str"/>
+      <x:c r="AS32" s="43" t="str"/>
       <x:c r="AT32" s="32" t="str"/>
       <x:c r="AU32" s="32" t="str"/>
       <x:c r="AV32" s="32" t="str"/>
-      <x:c r="AW32" s="33" t="str"/>
+      <x:c r="AW32" s="44" t="str"/>
       <x:c r="AX32" s="33" t="str"/>
       <x:c r="AY32" s="33" t="str"/>
       <x:c r="AZ32" s="33" t="str"/>
-      <x:c r="BA32" s="33" t="str">
+      <x:c r="BA32" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB32" s="33" t="str">
+      <x:c r="BB32" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC32" s="33" t="str">
+      <x:c r="BC32" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD32" s="33" t="str"/>
@@ -2915,58 +2926,58 @@
       <x:c r="E33" s="32" t="str"/>
       <x:c r="F33" s="32" t="str"/>
       <x:c r="G33" s="32" t="str"/>
-      <x:c r="H33" s="32" t="str"/>
-      <x:c r="I33" s="32" t="str"/>
-      <x:c r="J33" s="32" t="str"/>
-      <x:c r="K33" s="32" t="str"/>
-      <x:c r="L33" s="32" t="str"/>
-      <x:c r="M33" s="32" t="str"/>
-      <x:c r="N33" s="32" t="str"/>
-      <x:c r="O33" s="32" t="str"/>
-      <x:c r="P33" s="32" t="str"/>
-      <x:c r="Q33" s="32" t="str"/>
-      <x:c r="R33" s="32" t="str"/>
-      <x:c r="S33" s="32" t="str"/>
-      <x:c r="T33" s="32" t="str"/>
-      <x:c r="U33" s="32" t="str"/>
-      <x:c r="V33" s="32" t="str"/>
-      <x:c r="W33" s="32" t="str"/>
-      <x:c r="X33" s="32" t="str"/>
-      <x:c r="Y33" s="32" t="str"/>
-      <x:c r="Z33" s="32" t="str"/>
-      <x:c r="AA33" s="32" t="str"/>
-      <x:c r="AB33" s="32" t="str"/>
-      <x:c r="AC33" s="32" t="str"/>
-      <x:c r="AD33" s="32" t="str"/>
-      <x:c r="AE33" s="32" t="str"/>
-      <x:c r="AF33" s="32" t="str"/>
-      <x:c r="AG33" s="32" t="str"/>
-      <x:c r="AH33" s="32" t="str"/>
-      <x:c r="AI33" s="32" t="str"/>
-      <x:c r="AJ33" s="32" t="str"/>
-      <x:c r="AK33" s="32" t="str"/>
-      <x:c r="AL33" s="32" t="str"/>
-      <x:c r="AM33" s="32" t="str"/>
+      <x:c r="H33" s="43" t="str"/>
+      <x:c r="I33" s="43" t="str"/>
+      <x:c r="J33" s="43" t="str"/>
+      <x:c r="K33" s="43" t="str"/>
+      <x:c r="L33" s="43" t="str"/>
+      <x:c r="M33" s="43" t="str"/>
+      <x:c r="N33" s="43" t="str"/>
+      <x:c r="O33" s="43" t="str"/>
+      <x:c r="P33" s="43" t="str"/>
+      <x:c r="Q33" s="43" t="str"/>
+      <x:c r="R33" s="43" t="str"/>
+      <x:c r="S33" s="43" t="str"/>
+      <x:c r="T33" s="43" t="str"/>
+      <x:c r="U33" s="43" t="str"/>
+      <x:c r="V33" s="43" t="str"/>
+      <x:c r="W33" s="43" t="str"/>
+      <x:c r="X33" s="43" t="str"/>
+      <x:c r="Y33" s="43" t="str"/>
+      <x:c r="Z33" s="43" t="str"/>
+      <x:c r="AA33" s="43" t="str"/>
+      <x:c r="AB33" s="43" t="str"/>
+      <x:c r="AC33" s="43" t="str"/>
+      <x:c r="AD33" s="43" t="str"/>
+      <x:c r="AE33" s="43" t="str"/>
+      <x:c r="AF33" s="43" t="str"/>
+      <x:c r="AG33" s="43" t="str"/>
+      <x:c r="AH33" s="43" t="str"/>
+      <x:c r="AI33" s="43" t="str"/>
+      <x:c r="AJ33" s="43" t="str"/>
+      <x:c r="AK33" s="43" t="str"/>
+      <x:c r="AL33" s="43" t="str"/>
+      <x:c r="AM33" s="43" t="str"/>
       <x:c r="AN33" s="32" t="str"/>
-      <x:c r="AO33" s="32" t="str"/>
-      <x:c r="AP33" s="32" t="str"/>
+      <x:c r="AO33" s="43" t="str"/>
+      <x:c r="AP33" s="43" t="str"/>
       <x:c r="AQ33" s="32" t="str"/>
-      <x:c r="AR33" s="32" t="str"/>
-      <x:c r="AS33" s="32" t="str"/>
+      <x:c r="AR33" s="43" t="str"/>
+      <x:c r="AS33" s="43" t="str"/>
       <x:c r="AT33" s="32" t="str"/>
       <x:c r="AU33" s="32" t="str"/>
       <x:c r="AV33" s="32" t="str"/>
-      <x:c r="AW33" s="33" t="str"/>
+      <x:c r="AW33" s="44" t="str"/>
       <x:c r="AX33" s="33" t="str"/>
       <x:c r="AY33" s="33" t="str"/>
       <x:c r="AZ33" s="33" t="str"/>
-      <x:c r="BA33" s="33" t="str">
+      <x:c r="BA33" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB33" s="33" t="str">
+      <x:c r="BB33" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC33" s="33" t="str">
+      <x:c r="BC33" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD33" s="33" t="str"/>
@@ -2981,58 +2992,58 @@
       <x:c r="E34" s="32" t="str"/>
       <x:c r="F34" s="32" t="str"/>
       <x:c r="G34" s="32" t="str"/>
-      <x:c r="H34" s="32" t="str"/>
-      <x:c r="I34" s="32" t="str"/>
-      <x:c r="J34" s="32" t="str"/>
-      <x:c r="K34" s="32" t="str"/>
-      <x:c r="L34" s="32" t="str"/>
-      <x:c r="M34" s="32" t="str"/>
-      <x:c r="N34" s="32" t="str"/>
-      <x:c r="O34" s="32" t="str"/>
-      <x:c r="P34" s="32" t="str"/>
-      <x:c r="Q34" s="32" t="str"/>
-      <x:c r="R34" s="32" t="str"/>
-      <x:c r="S34" s="32" t="str"/>
-      <x:c r="T34" s="32" t="str"/>
-      <x:c r="U34" s="32" t="str"/>
-      <x:c r="V34" s="32" t="str"/>
-      <x:c r="W34" s="32" t="str"/>
-      <x:c r="X34" s="32" t="str"/>
-      <x:c r="Y34" s="32" t="str"/>
-      <x:c r="Z34" s="32" t="str"/>
-      <x:c r="AA34" s="32" t="str"/>
-      <x:c r="AB34" s="32" t="str"/>
-      <x:c r="AC34" s="32" t="str"/>
-      <x:c r="AD34" s="32" t="str"/>
-      <x:c r="AE34" s="32" t="str"/>
-      <x:c r="AF34" s="32" t="str"/>
-      <x:c r="AG34" s="32" t="str"/>
-      <x:c r="AH34" s="32" t="str"/>
-      <x:c r="AI34" s="32" t="str"/>
-      <x:c r="AJ34" s="32" t="str"/>
-      <x:c r="AK34" s="32" t="str"/>
-      <x:c r="AL34" s="32" t="str"/>
-      <x:c r="AM34" s="32" t="str"/>
+      <x:c r="H34" s="43" t="str"/>
+      <x:c r="I34" s="43" t="str"/>
+      <x:c r="J34" s="43" t="str"/>
+      <x:c r="K34" s="43" t="str"/>
+      <x:c r="L34" s="43" t="str"/>
+      <x:c r="M34" s="43" t="str"/>
+      <x:c r="N34" s="43" t="str"/>
+      <x:c r="O34" s="43" t="str"/>
+      <x:c r="P34" s="43" t="str"/>
+      <x:c r="Q34" s="43" t="str"/>
+      <x:c r="R34" s="43" t="str"/>
+      <x:c r="S34" s="43" t="str"/>
+      <x:c r="T34" s="43" t="str"/>
+      <x:c r="U34" s="43" t="str"/>
+      <x:c r="V34" s="43" t="str"/>
+      <x:c r="W34" s="43" t="str"/>
+      <x:c r="X34" s="43" t="str"/>
+      <x:c r="Y34" s="43" t="str"/>
+      <x:c r="Z34" s="43" t="str"/>
+      <x:c r="AA34" s="43" t="str"/>
+      <x:c r="AB34" s="43" t="str"/>
+      <x:c r="AC34" s="43" t="str"/>
+      <x:c r="AD34" s="43" t="str"/>
+      <x:c r="AE34" s="43" t="str"/>
+      <x:c r="AF34" s="43" t="str"/>
+      <x:c r="AG34" s="43" t="str"/>
+      <x:c r="AH34" s="43" t="str"/>
+      <x:c r="AI34" s="43" t="str"/>
+      <x:c r="AJ34" s="43" t="str"/>
+      <x:c r="AK34" s="43" t="str"/>
+      <x:c r="AL34" s="43" t="str"/>
+      <x:c r="AM34" s="43" t="str"/>
       <x:c r="AN34" s="32" t="str"/>
-      <x:c r="AO34" s="32" t="str"/>
-      <x:c r="AP34" s="32" t="str"/>
+      <x:c r="AO34" s="43" t="str"/>
+      <x:c r="AP34" s="43" t="str"/>
       <x:c r="AQ34" s="32" t="str"/>
-      <x:c r="AR34" s="32" t="str"/>
-      <x:c r="AS34" s="32" t="str"/>
+      <x:c r="AR34" s="43" t="str"/>
+      <x:c r="AS34" s="43" t="str"/>
       <x:c r="AT34" s="32" t="str"/>
       <x:c r="AU34" s="32" t="str"/>
       <x:c r="AV34" s="32" t="str"/>
-      <x:c r="AW34" s="33" t="str"/>
+      <x:c r="AW34" s="44" t="str"/>
       <x:c r="AX34" s="33" t="str"/>
       <x:c r="AY34" s="33" t="str"/>
       <x:c r="AZ34" s="33" t="str"/>
-      <x:c r="BA34" s="33" t="str">
+      <x:c r="BA34" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
-      <x:c r="BB34" s="33" t="str">
+      <x:c r="BB34" s="44" t="str">
         <x:v>در انتظار تصویر</x:v>
       </x:c>
-      <x:c r="BC34" s="33" t="str">
+      <x:c r="BC34" s="44" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
       <x:c r="BD34" s="33" t="str"/>
@@ -11407,15 +11418,6 @@
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Z5:Z34">
       <x:formula1>"بدون آماده‌سازی,ساده,متوسط"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" allowBlank="1" showDropDown="0" sqref="AA5:AA34">
-      <x:formula1>"بعد از کار,روز بارانی,قبل خواب"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" allowBlank="1" showDropDown="0" sqref="AB5:AB34">
-      <x:formula1>"بعد از کار,روز بارانی,قبل خواب"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" allowBlank="1" showDropDown="0" sqref="AC5:AC34">
-      <x:formula1>"بعد از کار,روز بارانی,قبل خواب"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showDropDown="0" sqref="AD5:AD34">
       <x:formula1>"داخل خانه,بیرون,رستوران,ماشین,مهمانی"</x:formula1>
@@ -11588,10 +11590,19 @@
       <x:formula1>0</x:formula1>
       <x:formula2>120</x:formula2>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="AA5:AA34">
+      <x:formula1>"بین وعده‌های غذایی,بعد از غذا,بین کارهای روزمره,قبل از خواب"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AB5:AB34">
+      <x:formula1>"بین وعده‌های غذایی,بعد از غذا,بین کارهای روزمره,قبل از خواب"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AC5:AC34">
+      <x:formula1>"بین وعده‌های غذایی,بعد از غذا,بین کارهای روزمره,قبل از خواب"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8b30dbac36745cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cac5ade932c402b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>